<commit_message>
Ingest CJB interview results (06/26) — hard gate cleared
- Store filled interview doc (CJB_Interview_Agenda_FILLED.docx)
- Roster: CJB -> INTERVIEWED/GATE CLEARED, STRONG; heating confirmed
  (90-95 C, 45min-1hr), 40 gal min / will do 55 gal, lead 3-4 days
- Pre-fill CJB Interview tab with captured answers + pass/follow-up flags
- MinBatch input -> 40 gal per CJB confirmation
- Open items flagged: price (Option A/B) not yet quoted; NDA on process

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inputs &amp; Assumptions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Split Scenarios" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Price Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="SNP Re-pricing Risk" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Supplier Roster" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CJB Interview" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs &amp; Assumptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Split Scenarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SNP Re-pricing Risk" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Roster" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJB Interview" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="DrumGal">'Inputs &amp; Assumptions'!$C$6</definedName>
@@ -335,7 +335,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -888,11 +890,11 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Corrected 2026-06-26: APV / Piedmont / Columbus all run from ~5 gal. A single drum (55 gal) is easily within a batch.</t>
+          <t>CJB confirmed (06/26): 40 gal min, MOQ 100 gal, will do 55 gal = 1 drum. A single drum is within a batch.</t>
         </is>
       </c>
     </row>
@@ -2034,32 +2036,32 @@
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>▶ INTERVIEWING (next call)</t>
+          <t>✔ INTERVIEWED 06/26 — GATE CLEARED</t>
         </is>
       </c>
       <c r="D7" s="29" t="inlineStr">
         <is>
-          <t>Confirm in interview</t>
+          <t>YES — holds 90-95 C for 45 min-1 hr (confirmed 06/26)</t>
         </is>
       </c>
       <c r="E7" s="29" t="inlineStr">
         <is>
-          <t>3 pilot systems + small-batch + scale-up</t>
+          <t>40 gal min; MOQ 100 gal, will do 55 gal (1 drum)</t>
         </is>
       </c>
       <c r="F7" s="29" t="inlineStr">
         <is>
-          <t>Excellent — pilot plants, courts start-ups</t>
-        </is>
-      </c>
-      <c r="G7" s="31" t="inlineStr">
-        <is>
-          <t>GOOD</t>
+          <t>Excellent — single drum OK; lab-batch available for qualification</t>
+        </is>
+      </c>
+      <c r="G7" s="32" t="inlineStr">
+        <is>
+          <t>STRONG</t>
         </is>
       </c>
       <c r="H7" s="29" t="inlineStr">
         <is>
-          <t>Has an EX-LONZA (Proxel) formulator on staff — directly relevant to your biocide. (229) 588-7200.</t>
+          <t>GATE CLEARED: jacketed 316L, agitation no fisheyes, cools to &lt;=40 C, prior HMW PVA experience. Lead 3-4 days or overnight; packaging flexible; ISO not required. Ex-Lonza (Proxel) formulator on staff. OPEN: NDA needed on process before full spec; PRICE not yet quoted (Option A/B).</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2683,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Fill the YELLOW cells during/after the call, save, and send the file back — I'll ingest it into the Roster &amp; model. Duplicate this tab (right-click &gt; Move or Copy) to reuse for APV / Columbus / Piedmont.</t>
+          <t>COMPLETED 2026-06-26 — HARD GATE CLEARED. Captured answers below; blanks = not covered on the call. OPEN: pricing (Option A/B) not yet quoted; NDA needed on process first. Duplicate this tab to reuse for APV / Columbus / Piedmont.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2723,7 @@
       </c>
       <c r="C6" s="36" t="inlineStr">
         <is>
-          <t>____</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="D6" s="37" t="n"/>
@@ -2775,10 +2777,14 @@
           <t>Holds 90-95 C cook 30-45 min? (Y/N)</t>
         </is>
       </c>
-      <c r="C11" s="40" t="inlineStr"/>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>YES — holds 45 min to 1 hr</t>
+        </is>
+      </c>
       <c r="D11" s="41" t="inlineStr">
         <is>
-          <t>HARD GATE</t>
+          <t>HARD GATE — CLEARED</t>
         </is>
       </c>
       <c r="E11" s="38" t="n"/>
@@ -2789,10 +2795,14 @@
           <t>Dissolves super-hydrolyzed HMW PVA? (Y/N)</t>
         </is>
       </c>
-      <c r="C12" s="40" t="inlineStr"/>
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>YES — has prior experience</t>
+        </is>
+      </c>
       <c r="D12" s="41" t="inlineStr">
         <is>
-          <t>HARD GATE</t>
+          <t>HARD GATE — CLEARED</t>
         </is>
       </c>
       <c r="E12" s="38" t="n"/>
@@ -2803,7 +2813,11 @@
           <t>Min batch size (gal)</t>
         </is>
       </c>
-      <c r="C13" s="40" t="inlineStr"/>
+      <c r="C13" s="40" t="inlineStr">
+        <is>
+          <t>40 gal min</t>
+        </is>
+      </c>
       <c r="D13" s="41" t="inlineStr">
         <is>
           <t>Inputs!MinBatch + shelf-life fit</t>
@@ -2817,7 +2831,11 @@
           <t>Will do partial / short batches? (Y/N)</t>
         </is>
       </c>
-      <c r="C14" s="40" t="inlineStr"/>
+      <c r="C14" s="40" t="inlineStr">
+        <is>
+          <t>YES — down to 40 gal; can lab-batch</t>
+        </is>
+      </c>
       <c r="D14" s="41" t="inlineStr">
         <is>
           <t>18-day shelf-life fit</t>
@@ -2831,7 +2849,11 @@
           <t>MOQ per order (drums)</t>
         </is>
       </c>
-      <c r="C15" s="40" t="inlineStr"/>
+      <c r="C15" s="40" t="inlineStr">
+        <is>
+          <t>100 gal (~2 drums); will do 55 gal (1 drum)</t>
+        </is>
+      </c>
       <c r="D15" s="41" t="inlineStr">
         <is>
           <t>Roster</t>
@@ -2845,7 +2867,11 @@
           <t>Price/drum — Option A, base ($)</t>
         </is>
       </c>
-      <c r="C16" s="40" t="inlineStr"/>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>NOT yet quoted (pending NDA + spec)</t>
+        </is>
+      </c>
       <c r="D16" s="41" t="inlineStr">
         <is>
           <t>Price Sensitivity input</t>
@@ -2859,7 +2885,11 @@
           <t>Price/drum — Option B, compounded ($)</t>
         </is>
       </c>
-      <c r="C17" s="40" t="inlineStr"/>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>NOT yet quoted</t>
+        </is>
+      </c>
       <c r="D17" s="41" t="inlineStr">
         <is>
           <t>Price Sensitivity input</t>
@@ -2873,7 +2903,11 @@
           <t>Lead time PO-&gt;delivery (days)</t>
         </is>
       </c>
-      <c r="C18" s="40" t="inlineStr"/>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>3-4 days, or overnight</t>
+        </is>
+      </c>
       <c r="D18" s="41" t="inlineStr">
         <is>
           <t>Roster</t>
@@ -2887,7 +2921,11 @@
           <t>Qualification sample qty &amp; cost</t>
         </is>
       </c>
-      <c r="C19" s="40" t="inlineStr"/>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>(not stated on call)</t>
+        </is>
+      </c>
       <c r="D19" s="41" t="inlineStr">
         <is>
           <t>Roster</t>
@@ -2901,7 +2939,11 @@
           <t>ISO 9001 / 13485? (which)</t>
         </is>
       </c>
-      <c r="C20" s="40" t="inlineStr"/>
+      <c r="C20" s="40" t="inlineStr">
+        <is>
+          <t>We don't require it</t>
+        </is>
+      </c>
       <c r="D20" s="41" t="inlineStr">
         <is>
           <t>Roster</t>
@@ -2915,7 +2957,11 @@
           <t>Prior PVA / HMW polymer experience? (Y/N)</t>
         </is>
       </c>
-      <c r="C21" s="40" t="inlineStr"/>
+      <c r="C21" s="40" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="D21" s="41" t="inlineStr">
         <is>
           <t>Roster</t>
@@ -2929,7 +2975,11 @@
           <t>NDA status</t>
         </is>
       </c>
-      <c r="C22" s="40" t="inlineStr"/>
+      <c r="C22" s="40" t="inlineStr">
+        <is>
+          <t>Needed on process before full spec shared</t>
+        </is>
+      </c>
       <c r="D22" s="41" t="inlineStr">
         <is>
           <t>Roster</t>
@@ -2983,8 +3033,16 @@
           <t>Can you heat a FULL batch to 90-95 C (194-203 F) and HOLD 30-45 min under steady agitation? Our cook requires it.</t>
         </is>
       </c>
-      <c r="C27" s="40" t="inlineStr"/>
-      <c r="D27" s="44" t="inlineStr"/>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>Yes — holds 45 min to 1 hr</t>
+        </is>
+      </c>
+      <c r="D27" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E27" s="38" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
@@ -2996,8 +3054,16 @@
           <t>Jacketed, temperature-controlled tank; 316L stainless contact surfaces?</t>
         </is>
       </c>
-      <c r="C28" s="40" t="inlineStr"/>
-      <c r="D28" s="44" t="inlineStr"/>
+      <c r="C28" s="40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D28" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E28" s="38" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
@@ -3009,8 +3075,16 @@
           <t>Variable-speed agitation able to dissolve high-MW super-hydrolyzed PVA with NO fisheyes / gels?</t>
         </is>
       </c>
-      <c r="C29" s="40" t="inlineStr"/>
-      <c r="D29" s="44" t="inlineStr"/>
+      <c r="C29" s="40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D29" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E29" s="38" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
@@ -3022,8 +3096,16 @@
           <t>Cooling capability to bring batch to &lt;=40 C?</t>
         </is>
       </c>
-      <c r="C30" s="40" t="inlineStr"/>
-      <c r="D30" s="44" t="inlineStr"/>
+      <c r="C30" s="40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D30" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E30" s="38" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
@@ -3035,8 +3117,16 @@
           <t>Have you dissolved PVA or similar high-MW water-soluble polymers before? Examples?</t>
         </is>
       </c>
-      <c r="C31" s="40" t="inlineStr"/>
-      <c r="D31" s="44" t="inlineStr"/>
+      <c r="C31" s="40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D31" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E31" s="38" t="n"/>
     </row>
     <row r="32">
@@ -3052,8 +3142,16 @@
           <t>Smallest batch you'll run? Will you do PARTIAL / short batches (~1-2 drums = 55-110 gal)?</t>
         </is>
       </c>
-      <c r="C33" s="40" t="inlineStr"/>
-      <c r="D33" s="44" t="inlineStr"/>
+      <c r="C33" s="40" t="inlineStr">
+        <is>
+          <t>40 gallons minimum</t>
+        </is>
+      </c>
+      <c r="D33" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E33" s="38" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
@@ -3065,8 +3163,16 @@
           <t>MOQ per order and standard batch size?</t>
         </is>
       </c>
-      <c r="C34" s="40" t="inlineStr"/>
-      <c r="D34" s="44" t="inlineStr"/>
+      <c r="C34" s="40" t="inlineStr">
+        <is>
+          <t>100 gal; could do 55 gal</t>
+        </is>
+      </c>
+      <c r="D34" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E34" s="38" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
@@ -3078,8 +3184,16 @@
           <t>Can you make-to-order on a ~weekly cadence? (18-day shelf life — we cannot stockpile.)</t>
         </is>
       </c>
-      <c r="C35" s="40" t="inlineStr"/>
-      <c r="D35" s="44" t="inlineStr"/>
+      <c r="C35" s="40" t="inlineStr">
+        <is>
+          <t>Yes — able to lab batch</t>
+        </is>
+      </c>
+      <c r="D35" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E35" s="38" t="n"/>
     </row>
     <row r="36">
@@ -3095,8 +3209,16 @@
           <t>Comfortable running OUR supplied process: charge water -&gt; add resin + NaCl + pigments -&gt; heat/hold 90-95 C -&gt; add Proxel BD20 hot in final 10 min -&gt; filter 200 micron -&gt; drum?</t>
         </is>
       </c>
-      <c r="C37" s="40" t="inlineStr"/>
-      <c r="D37" s="44" t="inlineStr"/>
+      <c r="C37" s="40" t="inlineStr">
+        <is>
+          <t>(not covered — confirm w/ full spec)</t>
+        </is>
+      </c>
+      <c r="D37" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E37" s="38" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
@@ -3108,8 +3230,16 @@
           <t>Filtration to 200 micron (100 mesh or finer)?</t>
         </is>
       </c>
-      <c r="C38" s="40" t="inlineStr"/>
-      <c r="D38" s="44" t="inlineStr"/>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>(not covered)</t>
+        </is>
+      </c>
+      <c r="D38" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E38" s="38" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
@@ -3121,8 +3251,16 @@
           <t>Your ex-Lonza formulator — any input on Proxel BD20 addition point / order / dosing?</t>
         </is>
       </c>
-      <c r="C39" s="40" t="inlineStr"/>
-      <c r="D39" s="44" t="inlineStr"/>
+      <c r="C39" s="40" t="inlineStr">
+        <is>
+          <t>(not covered)</t>
+        </is>
+      </c>
+      <c r="D39" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E39" s="38" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
@@ -3134,8 +3272,16 @@
           <t>Will you source raw materials to spec (Selvol S-1551F-D or equivalent) or do we supply the resin?</t>
         </is>
       </c>
-      <c r="C40" s="40" t="inlineStr"/>
-      <c r="D40" s="44" t="inlineStr"/>
+      <c r="C40" s="40" t="inlineStr">
+        <is>
+          <t>(not covered)</t>
+        </is>
+      </c>
+      <c r="D40" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E40" s="38" t="n"/>
     </row>
     <row r="41">
@@ -3151,8 +3297,16 @@
           <t>55-gallon drum fill? 275-gal IBC totes optional?</t>
         </is>
       </c>
-      <c r="C42" s="40" t="inlineStr"/>
-      <c r="D42" s="44" t="inlineStr"/>
+      <c r="C42" s="40" t="inlineStr">
+        <is>
+          <t>Packaging is flexible</t>
+        </is>
+      </c>
+      <c r="D42" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E42" s="38" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
@@ -3164,8 +3318,16 @@
           <t>Protect-from-freezing handling in shipping/storage?</t>
         </is>
       </c>
-      <c r="C43" s="40" t="inlineStr"/>
-      <c r="D43" s="44" t="inlineStr"/>
+      <c r="C43" s="40" t="inlineStr">
+        <is>
+          <t>(not covered)</t>
+        </is>
+      </c>
+      <c r="D43" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E43" s="38" t="n"/>
     </row>
     <row r="44" ht="30" customHeight="1">
@@ -3177,8 +3339,16 @@
           <t>Shipping from GA to us — lead time &amp; freight cost?</t>
         </is>
       </c>
-      <c r="C44" s="40" t="inlineStr"/>
-      <c r="D44" s="44" t="inlineStr"/>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>Lead time ~3-4 days, or overnight</t>
+        </is>
+      </c>
+      <c r="D44" s="44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="E44" s="38" t="n"/>
     </row>
     <row r="45">
@@ -3194,8 +3364,16 @@
           <t>CoC every shipment with lot#, production date, %TS, final pH, Brookfield viscosity (spindle #3, 10 RPM, 25 C)?</t>
         </is>
       </c>
-      <c r="C46" s="40" t="inlineStr"/>
-      <c r="D46" s="44" t="inlineStr"/>
+      <c r="C46" s="40" t="inlineStr">
+        <is>
+          <t>(not covered — confirm)</t>
+        </is>
+      </c>
+      <c r="D46" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E46" s="38" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
@@ -3207,8 +3385,16 @@
           <t>Typical batch-to-batch variability on viscosity &amp; pH for similar solutions?</t>
         </is>
       </c>
-      <c r="C47" s="40" t="inlineStr"/>
-      <c r="D47" s="44" t="inlineStr"/>
+      <c r="C47" s="40" t="inlineStr">
+        <is>
+          <t>(not covered)</t>
+        </is>
+      </c>
+      <c r="D47" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E47" s="38" t="n"/>
     </row>
     <row r="48" ht="30" customHeight="1">
@@ -3220,8 +3406,16 @@
           <t>Certifications — ISO 9001 minimum; ISO 13485 if available?</t>
         </is>
       </c>
-      <c r="C48" s="40" t="inlineStr"/>
-      <c r="D48" s="44" t="inlineStr"/>
+      <c r="C48" s="40" t="inlineStr">
+        <is>
+          <t>We don't require ISO certs</t>
+        </is>
+      </c>
+      <c r="D48" s="44" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E48" s="38" t="n"/>
     </row>
     <row r="49">
@@ -3237,8 +3431,16 @@
           <t>Quote BOTH Option A (base PVA solution) and Option B (full compounded w/ NaCl + pigments)?</t>
         </is>
       </c>
-      <c r="C50" s="40" t="inlineStr"/>
-      <c r="D50" s="44" t="inlineStr"/>
+      <c r="C50" s="40" t="inlineStr">
+        <is>
+          <t>(not yet — needs spec/NDA)</t>
+        </is>
+      </c>
+      <c r="D50" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E50" s="38" t="n"/>
     </row>
     <row r="51" ht="30" customHeight="1">
@@ -3250,8 +3452,16 @@
           <t>Per-drum pricing — we'll run this as a recurring rotation, ~1 drum/wk slice, ~30-38 drums/yr. Volume-agnostic per-drum quote?</t>
         </is>
       </c>
-      <c r="C51" s="40" t="inlineStr"/>
-      <c r="D51" s="44" t="inlineStr"/>
+      <c r="C51" s="40" t="inlineStr">
+        <is>
+          <t>(not yet quoted)</t>
+        </is>
+      </c>
+      <c r="D51" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E51" s="38" t="n"/>
     </row>
     <row r="52" ht="30" customHeight="1">
@@ -3263,8 +3473,16 @@
           <t>Lead time, qualification sample cost, and NDA needed before we share the full spec?</t>
         </is>
       </c>
-      <c r="C52" s="40" t="inlineStr"/>
-      <c r="D52" s="44" t="inlineStr"/>
+      <c r="C52" s="40" t="inlineStr">
+        <is>
+          <t>NDA needed on process</t>
+        </is>
+      </c>
+      <c r="D52" s="44" t="inlineStr">
+        <is>
+          <t>Follow-up</t>
+        </is>
+      </c>
       <c r="E52" s="38" t="n"/>
     </row>
     <row r="54">

</xml_diff>

<commit_message>
Add decided second-source allocation: 1 drum/week (~35%)
- New Inputs blocks: 2nd-source allocation (1 drum/wk = 52 drums/yr = ~35%)
  and a DECIDED PLAN cost summary (total, redundancy premium)
- SNP Re-pricing Risk tab re-based on the decided allocation (SNP retains ~98/yr)
- Split Scenarios highlight moved to the 33% row (closest to ~35%)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
@@ -25,11 +25,16 @@
     <definedName name="DrumsYr">'Inputs &amp; Assumptions'!$C$13</definedName>
     <definedName name="GalYr">'Inputs &amp; Assumptions'!$C$14</definedName>
     <definedName name="BaselineSpend">'Inputs &amp; Assumptions'!$C$15</definedName>
-    <definedName name="MinBatch">'Inputs &amp; Assumptions'!$C$18</definedName>
-    <definedName name="APVlow">'Inputs &amp; Assumptions'!$C$19</definedName>
-    <definedName name="APVlikely">'Inputs &amp; Assumptions'!$C$20</definedName>
-    <definedName name="APVhigh">'Inputs &amp; Assumptions'!$C$21</definedName>
-    <definedName name="SNPsurch">'Inputs &amp; Assumptions'!$C$24</definedName>
+    <definedName name="SrcDrumsWk">'Inputs &amp; Assumptions'!$C$18</definedName>
+    <definedName name="SrcDrumsYr">'Inputs &amp; Assumptions'!$C$19</definedName>
+    <definedName name="SrcSplit">'Inputs &amp; Assumptions'!$C$20</definedName>
+    <definedName name="SNPDrumsYr">'Inputs &amp; Assumptions'!$C$21</definedName>
+    <definedName name="MinBatch">'Inputs &amp; Assumptions'!$C$24</definedName>
+    <definedName name="APVlow">'Inputs &amp; Assumptions'!$C$25</definedName>
+    <definedName name="APVlikely">'Inputs &amp; Assumptions'!$C$26</definedName>
+    <definedName name="APVhigh">'Inputs &amp; Assumptions'!$C$27</definedName>
+    <definedName name="PlanTotal">'Inputs &amp; Assumptions'!$C$32</definedName>
+    <definedName name="SNPsurch">'Inputs &amp; Assumptions'!$C$37</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -220,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -250,6 +255,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -703,7 +714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E33"/>
+  <dimension ref="B2:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -877,7 +888,7 @@
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2) SECOND-SOURCE PRICE ASSUMPTIONS (placeholders until real quote)</t>
+          <t>1b) DECIDED SECOND-SOURCE ALLOCATION</t>
         </is>
       </c>
       <c r="C17" s="3" t="n"/>
@@ -886,70 +897,60 @@
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Min batch of best small-batch candidates (gal)</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="n">
-        <v>40</v>
+          <t>2nd-source allocation (drums / week)  &lt;-- DECISION</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>CJB confirmed (06/26): 40 gal min, MOQ 100 gal, will do 55 gal = 1 drum. A single drum is within a batch.</t>
+          <t>Plan (06/27): give the 2nd source ~1 drum/week.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>2nd-source price/drum - LOW (best case)</t>
-        </is>
-      </c>
-      <c r="C19" s="13">
-        <f>SNPdrum</f>
-        <v/>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Parity with SNP. Optimistic floor.</t>
-        </is>
+          <t>2nd-source drums / year</t>
+        </is>
+      </c>
+      <c r="C19" s="11">
+        <f>SrcDrumsWk*WeeksYr</f>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>2nd-source price/drum - LIKELY</t>
-        </is>
-      </c>
-      <c r="C20" s="13">
-        <f>ROUND(SNPdrum*1.5,2)</f>
+          <t>2nd-source share of total volume</t>
+        </is>
+      </c>
+      <c r="C20" s="14">
+        <f>SrcDrumsYr/DrumsYr</f>
         <v/>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>+50% small-batch premium. ADJUST when a real quote lands.</t>
+          <t>1 drum/wk is ~1/3 of total (~2.9 drums/wk).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>2nd-source price/drum - HIGH</t>
-        </is>
-      </c>
-      <c r="C21" s="13">
-        <f>ROUND(SNPdrum*2,2)</f>
-        <v/>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>+100% worst case.</t>
-        </is>
+          <t>SNP retains (drums / year)</t>
+        </is>
+      </c>
+      <c r="C21" s="11">
+        <f>DrumsYr-SrcDrumsYr</f>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>3) SNP RE-PRICING RISK (if SNP loses volume to a 2nd source)</t>
+          <t>2) SECOND-SOURCE PRICE ASSUMPTIONS (placeholders until real quote)</t>
         </is>
       </c>
       <c r="C23" s="3" t="n"/>
@@ -958,69 +959,210 @@
     <row r="24">
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>Min batch of best small-batch candidates (gal)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>CJB confirmed (06/26): 40 gal min, MOQ 100 gal, will do 55 gal = 1 drum. A single drum is within a batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>2nd-source price/drum - LOW (best case)</t>
+        </is>
+      </c>
+      <c r="C25" s="15">
+        <f>SNPdrum</f>
+        <v/>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Parity with SNP. Optimistic floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>2nd-source price/drum - LIKELY</t>
+        </is>
+      </c>
+      <c r="C26" s="15">
+        <f>ROUND(SNPdrum*1.5,2)</f>
+        <v/>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>+50% small-batch premium. ADJUST when a real quote lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>2nd-source price/drum - HIGH</t>
+        </is>
+      </c>
+      <c r="C27" s="15">
+        <f>ROUND(SNPdrum*2,2)</f>
+        <v/>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>+100% worst case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2b) DECIDED PLAN @ LIKELY price (1 drum/wk to 2nd source)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>2nd-source annual $ (@ likely)</t>
+        </is>
+      </c>
+      <c r="C30" s="9">
+        <f>SrcDrumsYr*APVlikely</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>SNP annual $ (retained)</t>
+        </is>
+      </c>
+      <c r="C31" s="9">
+        <f>SNPDrumsYr*SNPdrum</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL annual $ (decided plan)</t>
+        </is>
+      </c>
+      <c r="C32" s="9">
+        <f>SrcDrumsYr*APVlikely+SNPDrumsYr*SNPdrum</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Redundancy premium vs all-SNP ($)</t>
+        </is>
+      </c>
+      <c r="C33" s="9">
+        <f>PlanTotal-BaselineSpend</f>
+        <v/>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Cost of dual-sourcing at this allocation + price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Redundancy premium (%)</t>
+        </is>
+      </c>
+      <c r="C34" s="14">
+        <f>(PlanTotal-BaselineSpend)/BaselineSpend</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>3) SNP RE-PRICING RISK (if SNP loses volume to a 2nd source)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
           <t>SNP surcharge if volume reduced (%)</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
+      <c r="C37" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Set e.g. 10% to test whether SNP raises the rate on remaining drums. Used in scenarios.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="15" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="17" t="inlineStr">
         <is>
           <t>HOW TO USE:</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="6" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  - 'Split Scenarios': compare giving the 2nd source 0/10/20/25/33/50% of volume at the LIKELY price.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="6" t="inlineStr">
+    <row r="41">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  - 'Price Sensitivity': how total cost moves with the real per-drum quote x the split.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="6" t="inlineStr">
+    <row r="42">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  - 'SNP Re-pricing Risk': breakeven - how big an SNP surcharge erases the value of a 2nd source.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="6" t="inlineStr">
+    <row r="43">
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  - 'Supplier Roster': US candidates grouped by status + volume feasibility for a ~1 drum/wk slice.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="6" t="inlineStr">
+    <row r="44">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>DECIDED: fixed split ~20-25% to the 2nd source (~30-38 drums/yr), quoted per drum as a recurring rotation.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="6" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>GATING for any firm quote: viscosity target still pending from SNP CoA history.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="6" t="inlineStr">
+    <row r="46">
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>SECOND-SOURCE SLICE (~1 drum/wk) + 18-day shelf life =&gt; prefer suppliers with a SMALL min batch so you don't make more than ~2 drums you can use in time.</t>
         </is>
@@ -1067,301 +1209,301 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Split % to 2nd src</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>2nd-src drums/yr</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>SNP drums/yr</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>SNP $/drum
 (w/ surcharge)</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>2nd-src $/drum
 (Likely)</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>SNP annual $</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>2nd-src annual $</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>TOTAL annual $</t>
         </is>
       </c>
-      <c r="I4" s="16" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Δ vs all-SNP $</t>
         </is>
       </c>
-      <c r="J4" s="16" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>Δ %</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="20">
         <f>ROUND(DrumsYr*A5,1)</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="20">
         <f>ROUND(DrumsYr*(1-A5),1)</f>
         <v/>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="21">
         <f>IF(A5&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="21">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="21">
         <f>C5*D5</f>
         <v/>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="21">
         <f>B5*E5</f>
         <v/>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="21">
         <f>F5+G5</f>
         <v/>
       </c>
-      <c r="I5" s="19">
+      <c r="I5" s="21">
         <f>H5-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J5" s="20">
+      <c r="J5" s="22">
         <f>IF(BaselineSpend=0,0,I5/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="20">
         <f>ROUND(DrumsYr*A6,1)</f>
         <v/>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="20">
         <f>ROUND(DrumsYr*(1-A6),1)</f>
         <v/>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="21">
         <f>IF(A6&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="21">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="21">
         <f>C6*D6</f>
         <v/>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="21">
         <f>B6*E6</f>
         <v/>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="21">
         <f>F6+G6</f>
         <v/>
       </c>
-      <c r="I6" s="19">
+      <c r="I6" s="21">
         <f>H6-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J6" s="20">
+      <c r="J6" s="22">
         <f>IF(BaselineSpend=0,0,I6/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="20">
         <f>ROUND(DrumsYr*A7,1)</f>
         <v/>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="20">
         <f>ROUND(DrumsYr*(1-A7),1)</f>
         <v/>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="21">
         <f>IF(A7&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="21">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="21">
         <f>C7*D7</f>
         <v/>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="21">
         <f>B7*E7</f>
         <v/>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="21">
         <f>F7+G7</f>
         <v/>
       </c>
-      <c r="I7" s="23">
+      <c r="I7" s="21">
         <f>H7-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="22">
         <f>IF(BaselineSpend=0,0,I7/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="n">
+      <c r="A8" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="20">
         <f>ROUND(DrumsYr*A8,1)</f>
         <v/>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="20">
         <f>ROUND(DrumsYr*(1-A8),1)</f>
         <v/>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="21">
         <f>IF(A8&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="21">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="21">
         <f>C8*D8</f>
         <v/>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="21">
         <f>B8*E8</f>
         <v/>
       </c>
-      <c r="H8" s="23">
+      <c r="H8" s="21">
         <f>F8+G8</f>
         <v/>
       </c>
-      <c r="I8" s="23">
+      <c r="I8" s="21">
         <f>H8-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="22">
         <f>IF(BaselineSpend=0,0,I8/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="23" t="n">
         <v>0.33</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="24">
         <f>ROUND(DrumsYr*A9,1)</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="24">
         <f>ROUND(DrumsYr*(1-A9),1)</f>
         <v/>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="25">
         <f>IF(A9&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="25">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="25">
         <f>C9*D9</f>
         <v/>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="25">
         <f>B9*E9</f>
         <v/>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="25">
         <f>F9+G9</f>
         <v/>
       </c>
-      <c r="I9" s="19">
+      <c r="I9" s="25">
         <f>H9-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J9" s="20">
+      <c r="J9" s="26">
         <f>IF(BaselineSpend=0,0,I9/BaselineSpend)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="20">
         <f>ROUND(DrumsYr*A10,1)</f>
         <v/>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="20">
         <f>ROUND(DrumsYr*(1-A10),1)</f>
         <v/>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="21">
         <f>IF(A10&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="21">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="21">
         <f>C10*D10</f>
         <v/>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="21">
         <f>B10*E10</f>
         <v/>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="21">
         <f>F10+G10</f>
         <v/>
       </c>
-      <c r="I10" s="19">
+      <c r="I10" s="21">
         <f>H10-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J10" s="20">
+      <c r="J10" s="22">
         <f>IF(BaselineSpend=0,0,I10/BaselineSpend)</f>
         <v/>
       </c>
@@ -1369,7 +1511,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Highlighted rows (20% / 25%) = decided fixed-split range. 'Δ vs all-SNP' = annual cost of redundancy.</t>
+          <t>Highlighted row (33%) ~ the DECIDED plan: 1 drum/wk to the 2nd source = ~35%. Exact figures on Inputs '2b) DECIDED PLAN'. 'Δ vs all-SNP' = annual cost of redundancy.</t>
         </is>
       </c>
     </row>
@@ -1415,209 +1557,209 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>$/drum  ↓   Split →</t>
         </is>
       </c>
-      <c r="B4" s="26" t="n">
+      <c r="B4" s="28" t="n">
         <v>0.1</v>
       </c>
-      <c r="C4" s="26" t="n">
+      <c r="C4" s="28" t="n">
         <v>0.2</v>
       </c>
-      <c r="D4" s="26" t="n">
+      <c r="D4" s="28" t="n">
         <v>0.25</v>
       </c>
-      <c r="E4" s="26" t="n">
+      <c r="E4" s="28" t="n">
         <v>0.33</v>
       </c>
-      <c r="F4" s="26" t="n">
+      <c r="F4" s="28" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="n">
+      <c r="A5" s="15" t="n">
         <v>337.5</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="21">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A5</f>
         <v/>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="21">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A5</f>
         <v/>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="21">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A5</f>
         <v/>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="21">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A5</f>
         <v/>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="21">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="15" t="n">
         <v>400</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="21">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A6</f>
         <v/>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="21">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A6</f>
         <v/>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="21">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A6</f>
         <v/>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="21">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A6</f>
         <v/>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="21">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="15" t="n">
         <v>450</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="21">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A7</f>
         <v/>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="21">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A7</f>
         <v/>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="21">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A7</f>
         <v/>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="21">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A7</f>
         <v/>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="21">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="15" t="n">
         <v>506.25</v>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="21">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A8</f>
         <v/>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="21">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A8</f>
         <v/>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="21">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A8</f>
         <v/>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="21">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A8</f>
         <v/>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="21">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="15" t="n">
         <v>600</v>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="21">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A9</f>
         <v/>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="21">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A9</f>
         <v/>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="21">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A9</f>
         <v/>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="21">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A9</f>
         <v/>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="21">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="15" t="n">
         <v>675</v>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="21">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A10</f>
         <v/>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="21">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A10</f>
         <v/>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="21">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A10</f>
         <v/>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="21">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A10</f>
         <v/>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="21">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="15" t="n">
         <v>750</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="21">
         <f>DrumsYr*(1-0.1)*SNPdrum + DrumsYr*0.1*$A11</f>
         <v/>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="21">
         <f>DrumsYr*(1-0.2)*SNPdrum + DrumsYr*0.2*$A11</f>
         <v/>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="21">
         <f>DrumsYr*(1-0.25)*SNPdrum + DrumsYr*0.25*$A11</f>
         <v/>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="21">
         <f>DrumsYr*(1-0.33)*SNPdrum + DrumsYr*0.33*$A11</f>
         <v/>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="21">
         <f>DrumsYr*(1-0.5)*SNPdrum + DrumsYr*0.5*$A11</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Baseline all-SNP:</t>
         </is>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="30">
         <f>BaselineSpend</f>
         <v/>
       </c>
@@ -1667,217 +1809,217 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scenario: 25% to 2nd source at LIKELY price; SNP applies a surcharge on its remaining 75%.</t>
+          <t>Scenario: DECIDED PLAN (1 drum/wk to 2nd source, ~35%) at LIKELY price; SNP applies a surcharge on its retained ~98 drums/yr.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>SNP surcharge %</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>SNP $/drum</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>SNP annual (75%)</t>
-        </is>
-      </c>
-      <c r="D4" s="16" t="inlineStr">
-        <is>
-          <t>2nd-src annual (25%)</t>
-        </is>
-      </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>SNP annual (retained)</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>2nd-src annual (1 drum/wk)</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>TOTAL annual</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Δ vs all-SNP</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="n">
+      <c r="A5" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="B5" s="19">
+      <c r="B5" s="21">
         <f>SNPdrum*(1+A5)</f>
         <v/>
       </c>
-      <c r="C5" s="19">
-        <f>DrumsYr*(1-0.25)*B5</f>
-        <v/>
-      </c>
-      <c r="D5" s="19">
-        <f>DrumsYr*0.25*APVlikely</f>
-        <v/>
-      </c>
-      <c r="E5" s="19">
+      <c r="C5" s="21">
+        <f>SNPDrumsYr*B5</f>
+        <v/>
+      </c>
+      <c r="D5" s="21">
+        <f>SrcDrumsYr*APVlikely</f>
+        <v/>
+      </c>
+      <c r="E5" s="21">
         <f>C5+D5</f>
         <v/>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="21">
         <f>E5-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G5" s="29">
+      <c r="G5" s="31">
         <f>IF(F5&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F5,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="n">
+      <c r="A6" s="19" t="n">
         <v>0.05</v>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="21">
         <f>SNPdrum*(1+A6)</f>
         <v/>
       </c>
-      <c r="C6" s="19">
-        <f>DrumsYr*(1-0.25)*B6</f>
-        <v/>
-      </c>
-      <c r="D6" s="19">
-        <f>DrumsYr*0.25*APVlikely</f>
-        <v/>
-      </c>
-      <c r="E6" s="19">
+      <c r="C6" s="21">
+        <f>SNPDrumsYr*B6</f>
+        <v/>
+      </c>
+      <c r="D6" s="21">
+        <f>SrcDrumsYr*APVlikely</f>
+        <v/>
+      </c>
+      <c r="E6" s="21">
         <f>C6+D6</f>
         <v/>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="21">
         <f>E6-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G6" s="29">
+      <c r="G6" s="31">
         <f>IF(F6&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F6,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="n">
+      <c r="A7" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="B7" s="19">
+      <c r="B7" s="21">
         <f>SNPdrum*(1+A7)</f>
         <v/>
       </c>
-      <c r="C7" s="19">
-        <f>DrumsYr*(1-0.25)*B7</f>
-        <v/>
-      </c>
-      <c r="D7" s="19">
-        <f>DrumsYr*0.25*APVlikely</f>
-        <v/>
-      </c>
-      <c r="E7" s="19">
+      <c r="C7" s="21">
+        <f>SNPDrumsYr*B7</f>
+        <v/>
+      </c>
+      <c r="D7" s="21">
+        <f>SrcDrumsYr*APVlikely</f>
+        <v/>
+      </c>
+      <c r="E7" s="21">
         <f>C7+D7</f>
         <v/>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="21">
         <f>E7-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="31">
         <f>IF(F7&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F7,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n">
+      <c r="A8" s="19" t="n">
         <v>0.15</v>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="21">
         <f>SNPdrum*(1+A8)</f>
         <v/>
       </c>
-      <c r="C8" s="19">
-        <f>DrumsYr*(1-0.25)*B8</f>
-        <v/>
-      </c>
-      <c r="D8" s="19">
-        <f>DrumsYr*0.25*APVlikely</f>
-        <v/>
-      </c>
-      <c r="E8" s="19">
+      <c r="C8" s="21">
+        <f>SNPDrumsYr*B8</f>
+        <v/>
+      </c>
+      <c r="D8" s="21">
+        <f>SrcDrumsYr*APVlikely</f>
+        <v/>
+      </c>
+      <c r="E8" s="21">
         <f>C8+D8</f>
         <v/>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="21">
         <f>E8-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G8" s="29">
+      <c r="G8" s="31">
         <f>IF(F8&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F8,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="19" t="n">
         <v>0.2</v>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="21">
         <f>SNPdrum*(1+A9)</f>
         <v/>
       </c>
-      <c r="C9" s="19">
-        <f>DrumsYr*(1-0.25)*B9</f>
-        <v/>
-      </c>
-      <c r="D9" s="19">
-        <f>DrumsYr*0.25*APVlikely</f>
-        <v/>
-      </c>
-      <c r="E9" s="19">
+      <c r="C9" s="21">
+        <f>SNPDrumsYr*B9</f>
+        <v/>
+      </c>
+      <c r="D9" s="21">
+        <f>SrcDrumsYr*APVlikely</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
         <f>C9+D9</f>
         <v/>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="21">
         <f>E9-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="31">
         <f>IF(F9&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F9,"$#,##0"))</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n">
+      <c r="A10" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="21">
         <f>SNPdrum*(1+A10)</f>
         <v/>
       </c>
-      <c r="C10" s="19">
-        <f>DrumsYr*(1-0.25)*B10</f>
-        <v/>
-      </c>
-      <c r="D10" s="19">
-        <f>DrumsYr*0.25*APVlikely</f>
-        <v/>
-      </c>
-      <c r="E10" s="19">
+      <c r="C10" s="21">
+        <f>SNPDrumsYr*B10</f>
+        <v/>
+      </c>
+      <c r="D10" s="21">
+        <f>SrcDrumsYr*APVlikely</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
         <f>C10+D10</f>
         <v/>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="21">
         <f>E10-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G10" s="29">
+      <c r="G10" s="31">
         <f>IF(F10&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F10,"$#,##0"))</f>
         <v/>
       </c>
@@ -1933,703 +2075,703 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Holds 90-95 C?</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Min batch</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Small-batch + 18-day fit</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Volume feasibility</t>
         </is>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>ACTIVE SHORTLIST — right-sized for ~1 drum/wk + 18-day shelf life</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>APV Engineered Coatings</t>
         </is>
       </c>
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
         <is>
           <t>Akron, OH</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>▶ INTERVIEWING</t>
         </is>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="31" t="inlineStr">
         <is>
           <t>Re-confirm (verbal yes earlier; list flags as gating)</t>
         </is>
       </c>
-      <c r="E6" s="29" t="inlineStr">
+      <c r="E6" s="31" t="inlineStr">
         <is>
           <t>from 5 gal</t>
         </is>
       </c>
-      <c r="F6" s="29" t="inlineStr">
+      <c r="F6" s="31" t="inlineStr">
         <is>
           <t>Excellent — 5-gal floor easily makes 1 partial/full drum</t>
         </is>
       </c>
-      <c r="G6" s="31" t="inlineStr">
+      <c r="G6" s="33" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H6" s="29" t="inlineStr">
+      <c r="H6" s="31" t="inlineStr">
         <is>
           <t>Coatings house; pigment-dispersion specialty (good for your pigments); ISO 9001 / EPA-reg. CORRECTED: floor is ~5 gal, not 100. Gate to close in interview: 90-95 C hold.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>CJB Applied Technologies</t>
         </is>
       </c>
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>Valdosta, GA</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>✔ INTERVIEWED 06/26 — GATE CLEARED</t>
         </is>
       </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>YES — holds 90-95 C for 45 min-1 hr (confirmed 06/26)</t>
         </is>
       </c>
-      <c r="E7" s="29" t="inlineStr">
+      <c r="E7" s="31" t="inlineStr">
         <is>
           <t>40 gal min; MOQ 100 gal, will do 55 gal (1 drum)</t>
         </is>
       </c>
-      <c r="F7" s="29" t="inlineStr">
+      <c r="F7" s="31" t="inlineStr">
         <is>
           <t>Excellent — single drum OK; lab-batch available for qualification</t>
         </is>
       </c>
-      <c r="G7" s="32" t="inlineStr">
+      <c r="G7" s="34" t="inlineStr">
         <is>
           <t>STRONG</t>
         </is>
       </c>
-      <c r="H7" s="29" t="inlineStr">
+      <c r="H7" s="31" t="inlineStr">
         <is>
           <t>GATE CLEARED: jacketed 316L, agitation no fisheyes, cools to &lt;=40 C, prior HMW PVA experience. Lead 3-4 days or overnight; packaging flexible; ISO not required. Ex-Lonza (Proxel) formulator on staff. OPEN: NDA needed on process before full spec; PRICE not yet quoted (Option A/B).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>Piedmont Chemical</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>High Point, NC</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="31" t="inlineStr">
         <is>
           <t>Confirm 90-95 C</t>
         </is>
       </c>
-      <c r="E8" s="29" t="inlineStr">
+      <c r="E8" s="31" t="inlineStr">
         <is>
           <t>pilot reactors 5-100 gal</t>
         </is>
       </c>
-      <c r="F8" s="29" t="inlineStr">
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t>Good — 5-gal floor fits a single drum</t>
         </is>
       </c>
-      <c r="G8" s="31" t="inlineStr">
+      <c r="G8" s="33" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H8" s="29" t="inlineStr">
+      <c r="H8" s="31" t="inlineStr">
         <is>
           <t>UPGRADED from earlier 'too big': textile/PVA heritage = real PVA know-how; family-owned/agile. Best blend of PVA expertise + small-batch fit. (336) 885-5131.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Columbus Chemical (CCI)</t>
         </is>
       </c>
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>Columbus, WI / Phoenix, AZ</t>
         </is>
       </c>
-      <c r="C9" s="29" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="D9" s="29" t="inlineStr">
+      <c r="D9" s="31" t="inlineStr">
         <is>
           <t>Yes — heating/cooling</t>
         </is>
       </c>
-      <c r="E9" s="29" t="inlineStr">
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>20 L - 20,000 L (~5 gal floor)</t>
         </is>
       </c>
-      <c r="F9" s="29" t="inlineStr">
+      <c r="F9" s="31" t="inlineStr">
         <is>
           <t>Excellent — lowest floor, widest range</t>
         </is>
       </c>
-      <c r="G9" s="32" t="inlineStr">
+      <c r="G9" s="34" t="inlineStr">
         <is>
           <t>STRONG</t>
         </is>
       </c>
-      <c r="H9" s="29" t="inlineStr">
+      <c r="H9" s="31" t="inlineStr">
         <is>
           <t>In-house lab, ISO 9001. Widest batch range = least shelf-life waste; can scale if demand grows.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>CORECHEM</t>
         </is>
       </c>
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>Knoxville, TN</t>
         </is>
       </c>
-      <c r="C10" s="29" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="D10" s="29" t="inlineStr">
+      <c r="D10" s="31" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="E10" s="29" t="inlineStr">
+      <c r="E10" s="31" t="inlineStr">
         <is>
           <t>smallest tank ~250 gal (~4.5 drums)</t>
         </is>
       </c>
-      <c r="F10" s="29" t="inlineStr">
+      <c r="F10" s="31" t="inlineStr">
         <is>
           <t>CAUTION — 250-gal min may overshoot 18-day shelf life</t>
         </is>
       </c>
-      <c r="G10" s="33" t="inlineStr">
+      <c r="G10" s="35" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
       </c>
-      <c r="H10" s="29" t="inlineStr">
+      <c r="H10" s="31" t="inlineStr">
         <is>
           <t>Low-MOQ, start-up-friendly, family-owned. ASK about PARTIAL batches: a full 250-gal batch = ~4.5 drums but you can only use ~2 within 18 days.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Northstar Chemical</t>
         </is>
       </c>
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>Charlotte, NC</t>
         </is>
       </c>
-      <c r="C11" s="29" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>Backup</t>
         </is>
       </c>
-      <c r="D11" s="29" t="inlineStr">
+      <c r="D11" s="31" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="E11" s="29" t="inlineStr">
+      <c r="E11" s="31" t="inlineStr">
         <is>
           <t>unknown (small custom/toll)</t>
         </is>
       </c>
-      <c r="F11" s="29" t="inlineStr">
+      <c r="F11" s="31" t="inlineStr">
         <is>
           <t>Likely good — verify</t>
         </is>
       </c>
-      <c r="G11" s="31" t="inlineStr">
+      <c r="G11" s="33" t="inlineStr">
         <is>
           <t>LIKELY GOOD</t>
         </is>
       </c>
-      <c r="H11" s="29" t="inlineStr">
+      <c r="H11" s="31" t="inlineStr">
         <is>
           <t>Smaller dry-to-liquid custom/toll blender. (800) 570-0204.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>TECHNICAL ADVISOR — won't supply at this volume, but free expert call</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Sekisui Specialty Chemicals</t>
         </is>
       </c>
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>Calvert City, KY / Pasadena, TX</t>
         </is>
       </c>
-      <c r="C13" s="29" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>Advisor only</t>
         </is>
       </c>
-      <c r="D13" s="29" t="inlineStr">
+      <c r="D13" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E13" s="29" t="inlineStr">
+      <c r="E13" s="31" t="inlineStr">
         <is>
           <t>n/a (producer, bulk only)</t>
         </is>
       </c>
-      <c r="F13" s="29" t="inlineStr">
+      <c r="F13" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G13" s="34" t="inlineStr">
+      <c r="G13" s="36" t="inlineStr">
         <is>
           <t>N/A — advisor</t>
         </is>
       </c>
-      <c r="H13" s="29" t="inlineStr">
+      <c r="H13" s="31" t="inlineStr">
         <is>
           <t>Largest US PVOH (Selvol) producer. Free Tech Services call on grade selection + cook procedure. +1 855 436 8683.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>DROPPED — too large / MOQ mismatch for ~1 drum/wk</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Goulston Technologies</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t>Monroe, NC</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="31" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D15" s="29" t="inlineStr">
+      <c r="D15" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="29" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>large</t>
         </is>
       </c>
-      <c r="F15" s="29" t="inlineStr">
+      <c r="F15" s="31" t="inlineStr">
         <is>
           <t>Too big</t>
         </is>
       </c>
-      <c r="G15" s="35" t="inlineStr">
+      <c r="G15" s="37" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H15" s="29" t="inlineStr">
+      <c r="H15" s="31" t="inlineStr">
         <is>
           <t>Large textile chemical maker. 704-289-6464.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>3V Sigma USA</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t>Georgetown, SC</t>
         </is>
       </c>
-      <c r="C16" s="29" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D16" s="29" t="inlineStr">
+      <c r="D16" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="29" t="inlineStr">
+      <c r="E16" s="31" t="inlineStr">
         <is>
           <t>large</t>
         </is>
       </c>
-      <c r="F16" s="29" t="inlineStr">
+      <c r="F16" s="31" t="inlineStr">
         <is>
           <t>Too big</t>
         </is>
       </c>
-      <c r="G16" s="35" t="inlineStr">
+      <c r="G16" s="37" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H16" s="29" t="inlineStr">
+      <c r="H16" s="31" t="inlineStr">
         <is>
           <t>Large specialty chemical producer.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>Royal Chemical</t>
         </is>
       </c>
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>Twinsburg, OH (+5 sites)</t>
         </is>
       </c>
-      <c r="C17" s="29" t="inlineStr">
+      <c r="C17" s="31" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D17" s="29" t="inlineStr">
+      <c r="D17" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="29" t="inlineStr">
+      <c r="E17" s="31" t="inlineStr">
         <is>
           <t>220-gal liquid MOQ (~4 drums)</t>
         </is>
       </c>
-      <c r="F17" s="29" t="inlineStr">
+      <c r="F17" s="31" t="inlineStr">
         <is>
           <t>MOQ overshoots shelf life</t>
         </is>
       </c>
-      <c r="G17" s="35" t="inlineStr">
+      <c r="G17" s="37" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H17" s="29" t="inlineStr">
+      <c r="H17" s="31" t="inlineStr">
         <is>
           <t>220-gal min = ~4 drums = ~4 wks supply &gt; 18-day shelf life.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>Columbia Chemical</t>
         </is>
       </c>
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>Brunswick, OH</t>
         </is>
       </c>
-      <c r="C18" s="29" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D18" s="29" t="inlineStr">
+      <c r="D18" s="31" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E18" s="29" t="inlineStr">
+      <c r="E18" s="31" t="inlineStr">
         <is>
           <t>large</t>
         </is>
       </c>
-      <c r="F18" s="29" t="inlineStr">
+      <c r="F18" s="31" t="inlineStr">
         <is>
           <t>Too big / mismatch</t>
         </is>
       </c>
-      <c r="G18" s="35" t="inlineStr">
+      <c r="G18" s="37" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H18" s="29" t="inlineStr"/>
+      <c r="H18" s="31" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="32" t="inlineStr">
         <is>
           <t>ELIMINATED — failed the 90-95 C cook</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="29" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>ArroChem</t>
         </is>
       </c>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>Mt. Holly, NC</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C20" s="31" t="inlineStr">
         <is>
           <t>ELIMINATED</t>
         </is>
       </c>
-      <c r="D20" s="29" t="inlineStr">
+      <c r="D20" s="31" t="inlineStr">
         <is>
           <t>85 C ceiling — FAILS</t>
         </is>
       </c>
-      <c r="E20" s="29" t="inlineStr">
+      <c r="E20" s="31" t="inlineStr">
         <is>
           <t>55 gal (would have fit)</t>
         </is>
       </c>
-      <c r="F20" s="29" t="inlineStr">
+      <c r="F20" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G20" s="35" t="inlineStr">
+      <c r="G20" s="37" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H20" s="29" t="inlineStr">
+      <c r="H20" s="31" t="inlineStr">
         <is>
           <t>Volume fit was perfect (55-gal floor) but can't reach the 90-95 C cook.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="29" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>ILC Dover</t>
         </is>
       </c>
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
         <is>
           <t>Frederica, DE</t>
         </is>
       </c>
-      <c r="C21" s="29" t="inlineStr">
+      <c r="C21" s="31" t="inlineStr">
         <is>
           <t>ELIMINATED</t>
         </is>
       </c>
-      <c r="D21" s="29" t="inlineStr">
+      <c r="D21" s="31" t="inlineStr">
         <is>
           <t>Can't reach 95 C</t>
         </is>
       </c>
-      <c r="E21" s="29" t="inlineStr">
+      <c r="E21" s="31" t="inlineStr">
         <is>
           <t>n/a (equipment firm)</t>
         </is>
       </c>
-      <c r="F21" s="29" t="inlineStr">
+      <c r="F21" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G21" s="35" t="inlineStr">
+      <c r="G21" s="37" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H21" s="29" t="inlineStr">
+      <c r="H21" s="31" t="inlineStr">
         <is>
           <t>Wrong category (Ingersoll Rand containment/equipment) + heating fail. Close out.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="inlineStr">
+      <c r="A22" s="32" t="inlineStr">
         <is>
           <t>RAW RESIN PATH — reference only (supply Selvol resin, not the liquid blend)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Brenntag</t>
         </is>
       </c>
-      <c r="B23" s="29" t="inlineStr">
+      <c r="B23" s="31" t="inlineStr">
         <is>
           <t>US-wide</t>
         </is>
       </c>
-      <c r="C23" s="29" t="inlineStr">
+      <c r="C23" s="31" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="D23" s="29" t="inlineStr">
+      <c r="D23" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E23" s="29" t="inlineStr">
+      <c r="E23" s="31" t="inlineStr">
         <is>
           <t>single drums (core)</t>
         </is>
       </c>
-      <c r="F23" s="29" t="inlineStr">
+      <c r="F23" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G23" s="34" t="inlineStr">
+      <c r="G23" s="36" t="inlineStr">
         <is>
           <t>N/A — distributor</t>
         </is>
       </c>
-      <c r="H23" s="29" t="inlineStr">
+      <c r="H23" s="31" t="inlineStr">
         <is>
           <t>Already lists Sekisui Selvol → easiest source of genuine resin in drums if a blender needs it supplied.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="29" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>Tilley / Palmer Holland</t>
         </is>
       </c>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B24" s="31" t="inlineStr">
         <is>
           <t>Baltimore, MD / Westlake, OH</t>
         </is>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="D24" s="29" t="inlineStr">
+      <c r="D24" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E24" s="29" t="inlineStr">
+      <c r="E24" s="31" t="inlineStr">
         <is>
           <t>drums</t>
         </is>
       </c>
-      <c r="F24" s="29" t="inlineStr">
+      <c r="F24" s="31" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G24" s="34" t="inlineStr">
+      <c r="G24" s="36" t="inlineStr">
         <is>
           <t>N/A — distributor</t>
         </is>
       </c>
-      <c r="H24" s="29" t="inlineStr">
+      <c r="H24" s="31" t="inlineStr">
         <is>
           <t>Relationship-sized distributors; confirm they carry a PVA brand. Use only if sourcing raw resin.</t>
         </is>
@@ -2688,60 +2830,60 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="C4" s="36" t="inlineStr">
+      <c r="C4" s="38" t="inlineStr">
         <is>
           <t>CJB Applied Technologies (Valdosta, GA)</t>
         </is>
       </c>
-      <c r="D4" s="37" t="n"/>
-      <c r="E4" s="38" t="n"/>
+      <c r="D4" s="39" t="n"/>
+      <c r="E4" s="40" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Phone / contact</t>
         </is>
       </c>
-      <c r="C5" s="36" t="inlineStr">
+      <c r="C5" s="38" t="inlineStr">
         <is>
           <t>(229) 588-7200  /  ____</t>
         </is>
       </c>
-      <c r="D5" s="37" t="n"/>
-      <c r="E5" s="38" t="n"/>
+      <c r="D5" s="39" t="n"/>
+      <c r="E5" s="40" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Date of call</t>
         </is>
       </c>
-      <c r="C6" s="36" t="inlineStr">
+      <c r="C6" s="38" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="D6" s="37" t="n"/>
-      <c r="E6" s="38" t="n"/>
+      <c r="D6" s="39" t="n"/>
+      <c r="E6" s="40" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Interviewer</t>
         </is>
       </c>
-      <c r="C7" s="36" t="inlineStr">
+      <c r="C7" s="38" t="inlineStr">
         <is>
           <t>Oscar P</t>
         </is>
       </c>
-      <c r="D7" s="37" t="n"/>
-      <c r="E7" s="38" t="n"/>
+      <c r="D7" s="39" t="n"/>
+      <c r="E7" s="40" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
@@ -2754,238 +2896,238 @@
       <c r="E9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="39" t="inlineStr">
+      <c r="B10" s="41" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C10" s="39" t="inlineStr">
+      <c r="C10" s="41" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
-      <c r="D10" s="39" t="inlineStr">
+      <c r="D10" s="41" t="inlineStr">
         <is>
           <t>Maps to</t>
         </is>
       </c>
-      <c r="E10" s="38" t="n"/>
+      <c r="E10" s="40" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>Holds 90-95 C cook 30-45 min? (Y/N)</t>
         </is>
       </c>
-      <c r="C11" s="40" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
         <is>
           <t>YES — holds 45 min to 1 hr</t>
         </is>
       </c>
-      <c r="D11" s="41" t="inlineStr">
+      <c r="D11" s="43" t="inlineStr">
         <is>
           <t>HARD GATE — CLEARED</t>
         </is>
       </c>
-      <c r="E11" s="38" t="n"/>
+      <c r="E11" s="40" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="29" t="inlineStr">
+      <c r="B12" s="31" t="inlineStr">
         <is>
           <t>Dissolves super-hydrolyzed HMW PVA? (Y/N)</t>
         </is>
       </c>
-      <c r="C12" s="40" t="inlineStr">
+      <c r="C12" s="42" t="inlineStr">
         <is>
           <t>YES — has prior experience</t>
         </is>
       </c>
-      <c r="D12" s="41" t="inlineStr">
+      <c r="D12" s="43" t="inlineStr">
         <is>
           <t>HARD GATE — CLEARED</t>
         </is>
       </c>
-      <c r="E12" s="38" t="n"/>
+      <c r="E12" s="40" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>Min batch size (gal)</t>
         </is>
       </c>
-      <c r="C13" s="40" t="inlineStr">
+      <c r="C13" s="42" t="inlineStr">
         <is>
           <t>40 gal min</t>
         </is>
       </c>
-      <c r="D13" s="41" t="inlineStr">
+      <c r="D13" s="43" t="inlineStr">
         <is>
           <t>Inputs!MinBatch + shelf-life fit</t>
         </is>
       </c>
-      <c r="E13" s="38" t="n"/>
+      <c r="E13" s="40" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="31" t="inlineStr">
         <is>
           <t>Will do partial / short batches? (Y/N)</t>
         </is>
       </c>
-      <c r="C14" s="40" t="inlineStr">
+      <c r="C14" s="42" t="inlineStr">
         <is>
           <t>YES — down to 40 gal; can lab-batch</t>
         </is>
       </c>
-      <c r="D14" s="41" t="inlineStr">
+      <c r="D14" s="43" t="inlineStr">
         <is>
           <t>18-day shelf-life fit</t>
         </is>
       </c>
-      <c r="E14" s="38" t="n"/>
+      <c r="E14" s="40" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t>MOQ per order (drums)</t>
         </is>
       </c>
-      <c r="C15" s="40" t="inlineStr">
+      <c r="C15" s="42" t="inlineStr">
         <is>
           <t>100 gal (~2 drums); will do 55 gal (1 drum)</t>
         </is>
       </c>
-      <c r="D15" s="41" t="inlineStr">
+      <c r="D15" s="43" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E15" s="38" t="n"/>
+      <c r="E15" s="40" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t>Price/drum — Option A, base ($)</t>
         </is>
       </c>
-      <c r="C16" s="40" t="inlineStr">
+      <c r="C16" s="42" t="inlineStr">
         <is>
           <t>NOT yet quoted (pending NDA + spec)</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
+      <c r="D16" s="43" t="inlineStr">
         <is>
           <t>Price Sensitivity input</t>
         </is>
       </c>
-      <c r="E16" s="38" t="n"/>
+      <c r="E16" s="40" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>Price/drum — Option B, compounded ($)</t>
         </is>
       </c>
-      <c r="C17" s="40" t="inlineStr">
+      <c r="C17" s="42" t="inlineStr">
         <is>
           <t>NOT yet quoted</t>
         </is>
       </c>
-      <c r="D17" s="41" t="inlineStr">
+      <c r="D17" s="43" t="inlineStr">
         <is>
           <t>Price Sensitivity input</t>
         </is>
       </c>
-      <c r="E17" s="38" t="n"/>
+      <c r="E17" s="40" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="29" t="inlineStr">
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>Lead time PO-&gt;delivery (days)</t>
         </is>
       </c>
-      <c r="C18" s="40" t="inlineStr">
+      <c r="C18" s="42" t="inlineStr">
         <is>
           <t>3-4 days, or overnight</t>
         </is>
       </c>
-      <c r="D18" s="41" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E18" s="38" t="n"/>
+      <c r="E18" s="40" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="29" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
         <is>
           <t>Qualification sample qty &amp; cost</t>
         </is>
       </c>
-      <c r="C19" s="40" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
         <is>
           <t>(not stated on call)</t>
         </is>
       </c>
-      <c r="D19" s="41" t="inlineStr">
+      <c r="D19" s="43" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E19" s="38" t="n"/>
+      <c r="E19" s="40" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>ISO 9001 / 13485? (which)</t>
         </is>
       </c>
-      <c r="C20" s="40" t="inlineStr">
+      <c r="C20" s="42" t="inlineStr">
         <is>
           <t>We don't require it</t>
         </is>
       </c>
-      <c r="D20" s="41" t="inlineStr">
+      <c r="D20" s="43" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E20" s="38" t="n"/>
+      <c r="E20" s="40" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
         <is>
           <t>Prior PVA / HMW polymer experience? (Y/N)</t>
         </is>
       </c>
-      <c r="C21" s="40" t="inlineStr">
+      <c r="C21" s="42" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D21" s="41" t="inlineStr">
+      <c r="D21" s="43" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E21" s="38" t="n"/>
+      <c r="E21" s="40" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="29" t="inlineStr">
+      <c r="B22" s="31" t="inlineStr">
         <is>
           <t>NDA status</t>
         </is>
       </c>
-      <c r="C22" s="40" t="inlineStr">
+      <c r="C22" s="42" t="inlineStr">
         <is>
           <t>Needed on process before full spec shared</t>
         </is>
       </c>
-      <c r="D22" s="41" t="inlineStr">
+      <c r="D22" s="43" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E22" s="38" t="n"/>
+      <c r="E22" s="40" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
@@ -2998,492 +3140,492 @@
       <c r="E24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="39" t="inlineStr">
+      <c r="A25" s="41" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B25" s="39" t="inlineStr">
+      <c r="B25" s="41" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C25" s="39" t="inlineStr">
+      <c r="C25" s="41" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
-      <c r="D25" s="39" t="inlineStr">
+      <c r="D25" s="41" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
       </c>
-      <c r="E25" s="38" t="n"/>
+      <c r="E25" s="40" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="42" t="n"/>
+      <c r="A26" s="44" t="n"/>
       <c r="B26" s="4" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="43" t="n">
+      <c r="A27" s="45" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B27" s="31" t="inlineStr">
         <is>
           <t>Can you heat a FULL batch to 90-95 C (194-203 F) and HOLD 30-45 min under steady agitation? Our cook requires it.</t>
         </is>
       </c>
-      <c r="C27" s="40" t="inlineStr">
+      <c r="C27" s="42" t="inlineStr">
         <is>
           <t>Yes — holds 45 min to 1 hr</t>
         </is>
       </c>
-      <c r="D27" s="44" t="inlineStr">
+      <c r="D27" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E27" s="38" t="n"/>
+      <c r="E27" s="40" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="43" t="n">
+      <c r="A28" s="45" t="n">
         <v>2</v>
       </c>
-      <c r="B28" s="29" t="inlineStr">
+      <c r="B28" s="31" t="inlineStr">
         <is>
           <t>Jacketed, temperature-controlled tank; 316L stainless contact surfaces?</t>
         </is>
       </c>
-      <c r="C28" s="40" t="inlineStr">
+      <c r="C28" s="42" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D28" s="44" t="inlineStr">
+      <c r="D28" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E28" s="38" t="n"/>
+      <c r="E28" s="40" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="43" t="n">
+      <c r="A29" s="45" t="n">
         <v>3</v>
       </c>
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B29" s="31" t="inlineStr">
         <is>
           <t>Variable-speed agitation able to dissolve high-MW super-hydrolyzed PVA with NO fisheyes / gels?</t>
         </is>
       </c>
-      <c r="C29" s="40" t="inlineStr">
+      <c r="C29" s="42" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D29" s="44" t="inlineStr">
+      <c r="D29" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E29" s="38" t="n"/>
+      <c r="E29" s="40" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="43" t="n">
+      <c r="A30" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="B30" s="29" t="inlineStr">
+      <c r="B30" s="31" t="inlineStr">
         <is>
           <t>Cooling capability to bring batch to &lt;=40 C?</t>
         </is>
       </c>
-      <c r="C30" s="40" t="inlineStr">
+      <c r="C30" s="42" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D30" s="44" t="inlineStr">
+      <c r="D30" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E30" s="38" t="n"/>
+      <c r="E30" s="40" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="43" t="n">
+      <c r="A31" s="45" t="n">
         <v>5</v>
       </c>
-      <c r="B31" s="29" t="inlineStr">
+      <c r="B31" s="31" t="inlineStr">
         <is>
           <t>Have you dissolved PVA or similar high-MW water-soluble polymers before? Examples?</t>
         </is>
       </c>
-      <c r="C31" s="40" t="inlineStr">
+      <c r="C31" s="42" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D31" s="44" t="inlineStr">
+      <c r="D31" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E31" s="38" t="n"/>
+      <c r="E31" s="40" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="42" t="n"/>
+      <c r="A32" s="44" t="n"/>
       <c r="B32" s="4" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="43" t="n">
+      <c r="A33" s="45" t="n">
         <v>6</v>
       </c>
-      <c r="B33" s="29" t="inlineStr">
+      <c r="B33" s="31" t="inlineStr">
         <is>
           <t>Smallest batch you'll run? Will you do PARTIAL / short batches (~1-2 drums = 55-110 gal)?</t>
         </is>
       </c>
-      <c r="C33" s="40" t="inlineStr">
+      <c r="C33" s="42" t="inlineStr">
         <is>
           <t>40 gallons minimum</t>
         </is>
       </c>
-      <c r="D33" s="44" t="inlineStr">
+      <c r="D33" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E33" s="38" t="n"/>
+      <c r="E33" s="40" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="43" t="n">
+      <c r="A34" s="45" t="n">
         <v>7</v>
       </c>
-      <c r="B34" s="29" t="inlineStr">
+      <c r="B34" s="31" t="inlineStr">
         <is>
           <t>MOQ per order and standard batch size?</t>
         </is>
       </c>
-      <c r="C34" s="40" t="inlineStr">
+      <c r="C34" s="42" t="inlineStr">
         <is>
           <t>100 gal; could do 55 gal</t>
         </is>
       </c>
-      <c r="D34" s="44" t="inlineStr">
+      <c r="D34" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E34" s="38" t="n"/>
+      <c r="E34" s="40" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="43" t="n">
+      <c r="A35" s="45" t="n">
         <v>8</v>
       </c>
-      <c r="B35" s="29" t="inlineStr">
+      <c r="B35" s="31" t="inlineStr">
         <is>
           <t>Can you make-to-order on a ~weekly cadence? (18-day shelf life — we cannot stockpile.)</t>
         </is>
       </c>
-      <c r="C35" s="40" t="inlineStr">
+      <c r="C35" s="42" t="inlineStr">
         <is>
           <t>Yes — able to lab batch</t>
         </is>
       </c>
-      <c r="D35" s="44" t="inlineStr">
+      <c r="D35" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E35" s="38" t="n"/>
+      <c r="E35" s="40" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="42" t="n"/>
+      <c r="A36" s="44" t="n"/>
       <c r="B36" s="4" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="43" t="n">
+      <c r="A37" s="45" t="n">
         <v>9</v>
       </c>
-      <c r="B37" s="29" t="inlineStr">
+      <c r="B37" s="31" t="inlineStr">
         <is>
           <t>Comfortable running OUR supplied process: charge water -&gt; add resin + NaCl + pigments -&gt; heat/hold 90-95 C -&gt; add Proxel BD20 hot in final 10 min -&gt; filter 200 micron -&gt; drum?</t>
         </is>
       </c>
-      <c r="C37" s="40" t="inlineStr">
+      <c r="C37" s="42" t="inlineStr">
         <is>
           <t>(not covered — confirm w/ full spec)</t>
         </is>
       </c>
-      <c r="D37" s="44" t="inlineStr">
+      <c r="D37" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E37" s="38" t="n"/>
+      <c r="E37" s="40" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="43" t="n">
+      <c r="A38" s="45" t="n">
         <v>10</v>
       </c>
-      <c r="B38" s="29" t="inlineStr">
+      <c r="B38" s="31" t="inlineStr">
         <is>
           <t>Filtration to 200 micron (100 mesh or finer)?</t>
         </is>
       </c>
-      <c r="C38" s="40" t="inlineStr">
+      <c r="C38" s="42" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D38" s="44" t="inlineStr">
+      <c r="D38" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E38" s="38" t="n"/>
+      <c r="E38" s="40" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="43" t="n">
+      <c r="A39" s="45" t="n">
         <v>11</v>
       </c>
-      <c r="B39" s="29" t="inlineStr">
+      <c r="B39" s="31" t="inlineStr">
         <is>
           <t>Your ex-Lonza formulator — any input on Proxel BD20 addition point / order / dosing?</t>
         </is>
       </c>
-      <c r="C39" s="40" t="inlineStr">
+      <c r="C39" s="42" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D39" s="44" t="inlineStr">
+      <c r="D39" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E39" s="38" t="n"/>
+      <c r="E39" s="40" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="43" t="n">
+      <c r="A40" s="45" t="n">
         <v>12</v>
       </c>
-      <c r="B40" s="29" t="inlineStr">
+      <c r="B40" s="31" t="inlineStr">
         <is>
           <t>Will you source raw materials to spec (Selvol S-1551F-D or equivalent) or do we supply the resin?</t>
         </is>
       </c>
-      <c r="C40" s="40" t="inlineStr">
+      <c r="C40" s="42" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D40" s="44" t="inlineStr">
+      <c r="D40" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E40" s="38" t="n"/>
+      <c r="E40" s="40" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="42" t="n"/>
+      <c r="A41" s="44" t="n"/>
       <c r="B41" s="4" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="43" t="n">
+      <c r="A42" s="45" t="n">
         <v>13</v>
       </c>
-      <c r="B42" s="29" t="inlineStr">
+      <c r="B42" s="31" t="inlineStr">
         <is>
           <t>55-gallon drum fill? 275-gal IBC totes optional?</t>
         </is>
       </c>
-      <c r="C42" s="40" t="inlineStr">
+      <c r="C42" s="42" t="inlineStr">
         <is>
           <t>Packaging is flexible</t>
         </is>
       </c>
-      <c r="D42" s="44" t="inlineStr">
+      <c r="D42" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E42" s="38" t="n"/>
+      <c r="E42" s="40" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="43" t="n">
+      <c r="A43" s="45" t="n">
         <v>14</v>
       </c>
-      <c r="B43" s="29" t="inlineStr">
+      <c r="B43" s="31" t="inlineStr">
         <is>
           <t>Protect-from-freezing handling in shipping/storage?</t>
         </is>
       </c>
-      <c r="C43" s="40" t="inlineStr">
+      <c r="C43" s="42" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D43" s="44" t="inlineStr">
+      <c r="D43" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E43" s="38" t="n"/>
+      <c r="E43" s="40" t="n"/>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="43" t="n">
+      <c r="A44" s="45" t="n">
         <v>15</v>
       </c>
-      <c r="B44" s="29" t="inlineStr">
+      <c r="B44" s="31" t="inlineStr">
         <is>
           <t>Shipping from GA to us — lead time &amp; freight cost?</t>
         </is>
       </c>
-      <c r="C44" s="40" t="inlineStr">
+      <c r="C44" s="42" t="inlineStr">
         <is>
           <t>Lead time ~3-4 days, or overnight</t>
         </is>
       </c>
-      <c r="D44" s="44" t="inlineStr">
+      <c r="D44" s="46" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E44" s="38" t="n"/>
+      <c r="E44" s="40" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="42" t="n"/>
+      <c r="A45" s="44" t="n"/>
       <c r="B45" s="4" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="43" t="n">
+      <c r="A46" s="45" t="n">
         <v>16</v>
       </c>
-      <c r="B46" s="29" t="inlineStr">
+      <c r="B46" s="31" t="inlineStr">
         <is>
           <t>CoC every shipment with lot#, production date, %TS, final pH, Brookfield viscosity (spindle #3, 10 RPM, 25 C)?</t>
         </is>
       </c>
-      <c r="C46" s="40" t="inlineStr">
+      <c r="C46" s="42" t="inlineStr">
         <is>
           <t>(not covered — confirm)</t>
         </is>
       </c>
-      <c r="D46" s="44" t="inlineStr">
+      <c r="D46" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E46" s="38" t="n"/>
+      <c r="E46" s="40" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="43" t="n">
+      <c r="A47" s="45" t="n">
         <v>17</v>
       </c>
-      <c r="B47" s="29" t="inlineStr">
+      <c r="B47" s="31" t="inlineStr">
         <is>
           <t>Typical batch-to-batch variability on viscosity &amp; pH for similar solutions?</t>
         </is>
       </c>
-      <c r="C47" s="40" t="inlineStr">
+      <c r="C47" s="42" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D47" s="44" t="inlineStr">
+      <c r="D47" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E47" s="38" t="n"/>
+      <c r="E47" s="40" t="n"/>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="43" t="n">
+      <c r="A48" s="45" t="n">
         <v>18</v>
       </c>
-      <c r="B48" s="29" t="inlineStr">
+      <c r="B48" s="31" t="inlineStr">
         <is>
           <t>Certifications — ISO 9001 minimum; ISO 13485 if available?</t>
         </is>
       </c>
-      <c r="C48" s="40" t="inlineStr">
+      <c r="C48" s="42" t="inlineStr">
         <is>
           <t>We don't require ISO certs</t>
         </is>
       </c>
-      <c r="D48" s="44" t="inlineStr">
+      <c r="D48" s="46" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E48" s="38" t="n"/>
+      <c r="E48" s="40" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="42" t="n"/>
+      <c r="A49" s="44" t="n"/>
       <c r="B49" s="4" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="43" t="n">
+      <c r="A50" s="45" t="n">
         <v>19</v>
       </c>
-      <c r="B50" s="29" t="inlineStr">
+      <c r="B50" s="31" t="inlineStr">
         <is>
           <t>Quote BOTH Option A (base PVA solution) and Option B (full compounded w/ NaCl + pigments)?</t>
         </is>
       </c>
-      <c r="C50" s="40" t="inlineStr">
+      <c r="C50" s="42" t="inlineStr">
         <is>
           <t>(not yet — needs spec/NDA)</t>
         </is>
       </c>
-      <c r="D50" s="44" t="inlineStr">
+      <c r="D50" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E50" s="38" t="n"/>
+      <c r="E50" s="40" t="n"/>
     </row>
     <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="43" t="n">
+      <c r="A51" s="45" t="n">
         <v>20</v>
       </c>
-      <c r="B51" s="29" t="inlineStr">
+      <c r="B51" s="31" t="inlineStr">
         <is>
           <t>Per-drum pricing — we'll run this as a recurring rotation, ~1 drum/wk slice, ~30-38 drums/yr. Volume-agnostic per-drum quote?</t>
         </is>
       </c>
-      <c r="C51" s="40" t="inlineStr">
+      <c r="C51" s="42" t="inlineStr">
         <is>
           <t>(not yet quoted)</t>
         </is>
       </c>
-      <c r="D51" s="44" t="inlineStr">
+      <c r="D51" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E51" s="38" t="n"/>
+      <c r="E51" s="40" t="n"/>
     </row>
     <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="43" t="n">
+      <c r="A52" s="45" t="n">
         <v>21</v>
       </c>
-      <c r="B52" s="29" t="inlineStr">
+      <c r="B52" s="31" t="inlineStr">
         <is>
           <t>Lead time, qualification sample cost, and NDA needed before we share the full spec?</t>
         </is>
       </c>
-      <c r="C52" s="40" t="inlineStr">
+      <c r="C52" s="42" t="inlineStr">
         <is>
           <t>NDA needed on process</t>
         </is>
       </c>
-      <c r="D52" s="44" t="inlineStr">
+      <c r="D52" s="46" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E52" s="38" t="n"/>
+      <c r="E52" s="40" t="n"/>
     </row>
     <row r="54">
       <c r="B54" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Reframe as scenarios (nothing decided); add Cost-of-2nd-Source matrix
- Model: soften 'decided' labels to scenario language; add 'Cost of 2nd Source'
  tab — annual redundancy premium across allocation x 2nd-source price x SNP
  surcharge (incl. SNP-raises-price cases)
- Report & slides: replace decided-plan framing with scenario cost analysis;
  add the cost matrix and the 'SNP increase hits retained volume' insight

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Split Scenarios" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price Sensitivity" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SNP Re-pricing Risk" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Roster" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJB Interview" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost of 2nd Source" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supplier Roster" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJB Interview" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="DrumGal">'Inputs &amp; Assumptions'!$C$6</definedName>
@@ -48,7 +49,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,6 +90,10 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
@@ -126,6 +131,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00404040"/>
       </patternFill>
     </fill>
@@ -147,11 +157,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -225,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -287,18 +292,6 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -310,11 +303,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -328,21 +342,21 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -888,7 +902,7 @@
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>1b) DECIDED SECOND-SOURCE ALLOCATION</t>
+          <t>1b) SECOND-SOURCE ALLOCATION (scenario input — nothing decided)</t>
         </is>
       </c>
       <c r="C17" s="3" t="n"/>
@@ -897,7 +911,7 @@
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>2nd-source allocation (drums / week)  &lt;-- DECISION</t>
+          <t>2nd-source allocation (drums / week)  &lt;-- SCENARIO LEVER</t>
         </is>
       </c>
       <c r="C18" s="13" t="n">
@@ -905,7 +919,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Plan (06/27): give the 2nd source ~1 drum/week.</t>
+          <t>Scenario lever, NOT a decision. Change to explore. 1 drum/wk shown only as an example = ~35% of volume.</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1036,7 @@
     <row r="29">
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2b) DECIDED PLAN @ LIKELY price (1 drum/wk to 2nd source)</t>
+          <t>2b) SCENARIO RESULT (@ allocation above, likely price, SNP holds price)</t>
         </is>
       </c>
       <c r="C29" s="3" t="n"/>
@@ -1053,7 +1067,7 @@
     <row r="32">
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>TOTAL annual $ (decided plan)</t>
+          <t>TOTAL annual $ (this scenario)</t>
         </is>
       </c>
       <c r="C32" s="9">
@@ -1064,7 +1078,7 @@
     <row r="33">
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Redundancy premium vs all-SNP ($)</t>
+          <t>Cost of the 2nd source vs all-SNP ($)</t>
         </is>
       </c>
       <c r="C33" s="9">
@@ -1073,19 +1087,24 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Cost of dual-sourcing at this allocation + price.</t>
+          <t>Redundancy premium at this allocation + price (SNP price held).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Redundancy premium (%)</t>
+          <t>Cost of the 2nd source (%)</t>
         </is>
       </c>
       <c r="C34" s="14">
         <f>(PlanTotal-BaselineSpend)/BaselineSpend</f>
         <v/>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>See 'Cost of 2nd Source' tab for SNP-raises-price scenarios.</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1427,42 +1446,42 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
+      <c r="A9" s="19" t="n">
         <v>0.33</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="20">
         <f>ROUND(DrumsYr*A9,1)</f>
         <v/>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="20">
         <f>ROUND(DrumsYr*(1-A9),1)</f>
         <v/>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="21">
         <f>IF(A9&gt;0,SNPdrum*(1+SNPsurch),SNPdrum)</f>
         <v/>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="21">
         <f>APVlikely</f>
         <v/>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="21">
         <f>C9*D9</f>
         <v/>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="21">
         <f>B9*E9</f>
         <v/>
       </c>
-      <c r="H9" s="25">
+      <c r="H9" s="21">
         <f>F9+G9</f>
         <v/>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="21">
         <f>H9-BaselineSpend</f>
         <v/>
       </c>
-      <c r="J9" s="26">
+      <c r="J9" s="22">
         <f>IF(BaselineSpend=0,0,I9/BaselineSpend)</f>
         <v/>
       </c>
@@ -1511,7 +1530,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Highlighted row (33%) ~ the DECIDED plan: 1 drum/wk to the 2nd source = ~35%. Exact figures on Inputs '2b) DECIDED PLAN'. 'Δ vs all-SNP' = annual cost of redundancy.</t>
+          <t>Each row is a SCENARIO (nothing decided). 'Δ vs all-SNP' = the annual cost of keeping a second source at that split, assuming SNP HOLDS its price. For SNP-raises-price cases see the 'SNP Re-pricing Risk' and 'Cost of 2nd Source' tabs.</t>
         </is>
       </c>
     </row>
@@ -1557,24 +1576,24 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>$/drum  ↓   Split →</t>
         </is>
       </c>
-      <c r="B4" s="28" t="n">
+      <c r="B4" s="24" t="n">
         <v>0.1</v>
       </c>
-      <c r="C4" s="28" t="n">
+      <c r="C4" s="24" t="n">
         <v>0.2</v>
       </c>
-      <c r="D4" s="28" t="n">
+      <c r="D4" s="24" t="n">
         <v>0.25</v>
       </c>
-      <c r="E4" s="28" t="n">
+      <c r="E4" s="24" t="n">
         <v>0.33</v>
       </c>
-      <c r="F4" s="28" t="n">
+      <c r="F4" s="24" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -1754,12 +1773,12 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>Baseline all-SNP:</t>
         </is>
       </c>
-      <c r="C13" s="30">
+      <c r="C13" s="26">
         <f>BaselineSpend</f>
         <v/>
       </c>
@@ -1809,7 +1828,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Scenario: DECIDED PLAN (1 drum/wk to 2nd source, ~35%) at LIKELY price; SNP applies a surcharge on its retained ~98 drums/yr.</t>
+          <t>Scenario: 2nd source = the allocation set on Inputs (example 1 drum/wk ~35%) at LIKELY price; SNP applies a surcharge on its retained volume. Nothing decided.</t>
         </is>
       </c>
     </row>
@@ -1874,7 +1893,7 @@
         <f>E5-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="27">
         <f>IF(F5&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F5,"$#,##0"))</f>
         <v/>
       </c>
@@ -1903,7 +1922,7 @@
         <f>E6-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="27">
         <f>IF(F6&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F6,"$#,##0"))</f>
         <v/>
       </c>
@@ -1932,7 +1951,7 @@
         <f>E7-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="27">
         <f>IF(F7&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F7,"$#,##0"))</f>
         <v/>
       </c>
@@ -1961,7 +1980,7 @@
         <f>E8-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G8" s="31">
+      <c r="G8" s="27">
         <f>IF(F8&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F8,"$#,##0"))</f>
         <v/>
       </c>
@@ -1990,7 +2009,7 @@
         <f>E9-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G9" s="31">
+      <c r="G9" s="27">
         <f>IF(F9&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F9,"$#,##0"))</f>
         <v/>
       </c>
@@ -2019,7 +2038,7 @@
         <f>E10-BaselineSpend</f>
         <v/>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="27">
         <f>IF(F10&lt;=0,"Cheaper than baseline","Redundancy premium: "&amp;TEXT(F10,"$#,##0"))</f>
         <v/>
       </c>
@@ -2042,6 +2061,522 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cost of Keeping a Second Source — Scenario Matrix</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Annual PREMIUM over the all-SNP baseline (the extra you pay for redundancy). Auto-updates from Inputs. Nothing here is decided.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Premium = baseline x [ allocation x (2nd-source price premium) + retained x (SNP surcharge) ].   Note: 1 drum/wk ~= 35% of volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>SNP price increase on retained volume:  +0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Allocation to 2nd source  /  2nd-source price</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>2nd @ parity</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>2nd +25%</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>2nd +50%</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>2nd +100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="30" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="B7" s="31">
+        <f>BaselineSpend*(0.1*0.0+(1-0.1)*0.0)</f>
+        <v/>
+      </c>
+      <c r="C7" s="32">
+        <f>BaselineSpend*(0.1*0.25+(1-0.1)*0.0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="33">
+        <f>BaselineSpend*(0.1*0.5+(1-0.1)*0.0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="34">
+        <f>BaselineSpend*(0.1*1.0+(1-0.1)*0.0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="B8" s="31">
+        <f>BaselineSpend*(0.2*0.0+(1-0.2)*0.0)</f>
+        <v/>
+      </c>
+      <c r="C8" s="32">
+        <f>BaselineSpend*(0.2*0.25+(1-0.2)*0.0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="33">
+        <f>BaselineSpend*(0.2*0.5+(1-0.2)*0.0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="34">
+        <f>BaselineSpend*(0.2*1.0+(1-0.2)*0.0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="B9" s="31">
+        <f>BaselineSpend*(0.25*0.0+(1-0.25)*0.0)</f>
+        <v/>
+      </c>
+      <c r="C9" s="32">
+        <f>BaselineSpend*(0.25*0.25+(1-0.25)*0.0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="33">
+        <f>BaselineSpend*(0.25*0.5+(1-0.25)*0.0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="34">
+        <f>BaselineSpend*(0.25*1.0+(1-0.25)*0.0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>35% (~1 drum/wk)</t>
+        </is>
+      </c>
+      <c r="B10" s="31">
+        <f>BaselineSpend*(0.35*0.0+(1-0.35)*0.0)</f>
+        <v/>
+      </c>
+      <c r="C10" s="32">
+        <f>BaselineSpend*(0.35*0.25+(1-0.35)*0.0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="33">
+        <f>BaselineSpend*(0.35*0.5+(1-0.35)*0.0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="34">
+        <f>BaselineSpend*(0.35*1.0+(1-0.35)*0.0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="B11" s="31">
+        <f>BaselineSpend*(0.5*0.0+(1-0.5)*0.0)</f>
+        <v/>
+      </c>
+      <c r="C11" s="32">
+        <f>BaselineSpend*(0.5*0.25+(1-0.5)*0.0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="33">
+        <f>BaselineSpend*(0.5*0.5+(1-0.5)*0.0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="34">
+        <f>BaselineSpend*(0.5*1.0+(1-0.5)*0.0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>SNP price increase on retained volume:  +10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Allocation to 2nd source  /  2nd-source price</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>2nd @ parity</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>2nd +25%</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>2nd +50%</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="inlineStr">
+        <is>
+          <t>2nd +100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="B15" s="31">
+        <f>BaselineSpend*(0.1*0.0+(1-0.1)*0.1)</f>
+        <v/>
+      </c>
+      <c r="C15" s="32">
+        <f>BaselineSpend*(0.1*0.25+(1-0.1)*0.1)</f>
+        <v/>
+      </c>
+      <c r="D15" s="33">
+        <f>BaselineSpend*(0.1*0.5+(1-0.1)*0.1)</f>
+        <v/>
+      </c>
+      <c r="E15" s="34">
+        <f>BaselineSpend*(0.1*1.0+(1-0.1)*0.1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="B16" s="31">
+        <f>BaselineSpend*(0.2*0.0+(1-0.2)*0.1)</f>
+        <v/>
+      </c>
+      <c r="C16" s="32">
+        <f>BaselineSpend*(0.2*0.25+(1-0.2)*0.1)</f>
+        <v/>
+      </c>
+      <c r="D16" s="33">
+        <f>BaselineSpend*(0.2*0.5+(1-0.2)*0.1)</f>
+        <v/>
+      </c>
+      <c r="E16" s="34">
+        <f>BaselineSpend*(0.2*1.0+(1-0.2)*0.1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="B17" s="31">
+        <f>BaselineSpend*(0.25*0.0+(1-0.25)*0.1)</f>
+        <v/>
+      </c>
+      <c r="C17" s="32">
+        <f>BaselineSpend*(0.25*0.25+(1-0.25)*0.1)</f>
+        <v/>
+      </c>
+      <c r="D17" s="33">
+        <f>BaselineSpend*(0.25*0.5+(1-0.25)*0.1)</f>
+        <v/>
+      </c>
+      <c r="E17" s="34">
+        <f>BaselineSpend*(0.25*1.0+(1-0.25)*0.1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>35% (~1 drum/wk)</t>
+        </is>
+      </c>
+      <c r="B18" s="31">
+        <f>BaselineSpend*(0.35*0.0+(1-0.35)*0.1)</f>
+        <v/>
+      </c>
+      <c r="C18" s="32">
+        <f>BaselineSpend*(0.35*0.25+(1-0.35)*0.1)</f>
+        <v/>
+      </c>
+      <c r="D18" s="33">
+        <f>BaselineSpend*(0.35*0.5+(1-0.35)*0.1)</f>
+        <v/>
+      </c>
+      <c r="E18" s="34">
+        <f>BaselineSpend*(0.35*1.0+(1-0.35)*0.1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="B19" s="31">
+        <f>BaselineSpend*(0.5*0.0+(1-0.5)*0.1)</f>
+        <v/>
+      </c>
+      <c r="C19" s="32">
+        <f>BaselineSpend*(0.5*0.25+(1-0.5)*0.1)</f>
+        <v/>
+      </c>
+      <c r="D19" s="33">
+        <f>BaselineSpend*(0.5*0.5+(1-0.5)*0.1)</f>
+        <v/>
+      </c>
+      <c r="E19" s="34">
+        <f>BaselineSpend*(0.5*1.0+(1-0.5)*0.1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>SNP price increase on retained volume:  +20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Allocation to 2nd source  /  2nd-source price</t>
+        </is>
+      </c>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>2nd @ parity</t>
+        </is>
+      </c>
+      <c r="C22" s="29" t="inlineStr">
+        <is>
+          <t>2nd +25%</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="inlineStr">
+        <is>
+          <t>2nd +50%</t>
+        </is>
+      </c>
+      <c r="E22" s="29" t="inlineStr">
+        <is>
+          <t>2nd +100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="B23" s="31">
+        <f>BaselineSpend*(0.1*0.0+(1-0.1)*0.2)</f>
+        <v/>
+      </c>
+      <c r="C23" s="32">
+        <f>BaselineSpend*(0.1*0.25+(1-0.1)*0.2)</f>
+        <v/>
+      </c>
+      <c r="D23" s="33">
+        <f>BaselineSpend*(0.1*0.5+(1-0.1)*0.2)</f>
+        <v/>
+      </c>
+      <c r="E23" s="34">
+        <f>BaselineSpend*(0.1*1.0+(1-0.1)*0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="B24" s="31">
+        <f>BaselineSpend*(0.2*0.0+(1-0.2)*0.2)</f>
+        <v/>
+      </c>
+      <c r="C24" s="32">
+        <f>BaselineSpend*(0.2*0.25+(1-0.2)*0.2)</f>
+        <v/>
+      </c>
+      <c r="D24" s="33">
+        <f>BaselineSpend*(0.2*0.5+(1-0.2)*0.2)</f>
+        <v/>
+      </c>
+      <c r="E24" s="34">
+        <f>BaselineSpend*(0.2*1.0+(1-0.2)*0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="B25" s="31">
+        <f>BaselineSpend*(0.25*0.0+(1-0.25)*0.2)</f>
+        <v/>
+      </c>
+      <c r="C25" s="32">
+        <f>BaselineSpend*(0.25*0.25+(1-0.25)*0.2)</f>
+        <v/>
+      </c>
+      <c r="D25" s="33">
+        <f>BaselineSpend*(0.25*0.5+(1-0.25)*0.2)</f>
+        <v/>
+      </c>
+      <c r="E25" s="34">
+        <f>BaselineSpend*(0.25*1.0+(1-0.25)*0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="30" t="inlineStr">
+        <is>
+          <t>35% (~1 drum/wk)</t>
+        </is>
+      </c>
+      <c r="B26" s="31">
+        <f>BaselineSpend*(0.35*0.0+(1-0.35)*0.2)</f>
+        <v/>
+      </c>
+      <c r="C26" s="32">
+        <f>BaselineSpend*(0.35*0.25+(1-0.35)*0.2)</f>
+        <v/>
+      </c>
+      <c r="D26" s="33">
+        <f>BaselineSpend*(0.35*0.5+(1-0.35)*0.2)</f>
+        <v/>
+      </c>
+      <c r="E26" s="34">
+        <f>BaselineSpend*(0.35*1.0+(1-0.35)*0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="30" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="B27" s="31">
+        <f>BaselineSpend*(0.5*0.0+(1-0.5)*0.2)</f>
+        <v/>
+      </c>
+      <c r="C27" s="32">
+        <f>BaselineSpend*(0.5*0.25+(1-0.5)*0.2)</f>
+        <v/>
+      </c>
+      <c r="D27" s="33">
+        <f>BaselineSpend*(0.5*0.5+(1-0.5)*0.2)</f>
+        <v/>
+      </c>
+      <c r="E27" s="34">
+        <f>BaselineSpend*(0.5*1.0+(1-0.5)*0.2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="35" t="inlineStr">
+        <is>
+          <t>KEY INSIGHT: an SNP increase hits your LARGER retained volume, so it can cost MORE than the 2nd-source premium itself — compare the +0% block to the +10%/+20% blocks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t>Baseline (all-SNP) for reference:</t>
+        </is>
+      </c>
+      <c r="B30" s="26">
+        <f>BaselineSpend</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2117,661 +2652,661 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>ACTIVE SHORTLIST — right-sized for ~1 drum/wk + 18-day shelf life</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>APV Engineered Coatings</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>Akron, OH</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>▶ INTERVIEWING</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Re-confirm (verbal yes earlier; list flags as gating)</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>from 5 gal</t>
         </is>
       </c>
-      <c r="F6" s="31" t="inlineStr">
+      <c r="F6" s="27" t="inlineStr">
         <is>
           <t>Excellent — 5-gal floor easily makes 1 partial/full drum</t>
         </is>
       </c>
-      <c r="G6" s="33" t="inlineStr">
+      <c r="G6" s="37" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H6" s="31" t="inlineStr">
+      <c r="H6" s="27" t="inlineStr">
         <is>
           <t>Coatings house; pigment-dispersion specialty (good for your pigments); ISO 9001 / EPA-reg. CORRECTED: floor is ~5 gal, not 100. Gate to close in interview: 90-95 C hold.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>CJB Applied Technologies</t>
         </is>
       </c>
-      <c r="B7" s="31" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>Valdosta, GA</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>✔ INTERVIEWED 06/26 — GATE CLEARED</t>
         </is>
       </c>
-      <c r="D7" s="31" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>YES — holds 90-95 C for 45 min-1 hr (confirmed 06/26)</t>
         </is>
       </c>
-      <c r="E7" s="31" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>40 gal min; MOQ 100 gal, will do 55 gal (1 drum)</t>
         </is>
       </c>
-      <c r="F7" s="31" t="inlineStr">
+      <c r="F7" s="27" t="inlineStr">
         <is>
           <t>Excellent — single drum OK; lab-batch available for qualification</t>
         </is>
       </c>
-      <c r="G7" s="34" t="inlineStr">
+      <c r="G7" s="38" t="inlineStr">
         <is>
           <t>STRONG</t>
         </is>
       </c>
-      <c r="H7" s="31" t="inlineStr">
+      <c r="H7" s="27" t="inlineStr">
         <is>
           <t>GATE CLEARED: jacketed 316L, agitation no fisheyes, cools to &lt;=40 C, prior HMW PVA experience. Lead 3-4 days or overnight; packaging flexible; ISO not required. Ex-Lonza (Proxel) formulator on staff. OPEN: NDA needed on process before full spec; PRICE not yet quoted (Option A/B).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Piedmont Chemical</t>
         </is>
       </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>High Point, NC</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="D8" s="31" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>Confirm 90-95 C</t>
         </is>
       </c>
-      <c r="E8" s="31" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>pilot reactors 5-100 gal</t>
         </is>
       </c>
-      <c r="F8" s="31" t="inlineStr">
+      <c r="F8" s="27" t="inlineStr">
         <is>
           <t>Good — 5-gal floor fits a single drum</t>
         </is>
       </c>
-      <c r="G8" s="33" t="inlineStr">
+      <c r="G8" s="37" t="inlineStr">
         <is>
           <t>GOOD</t>
         </is>
       </c>
-      <c r="H8" s="31" t="inlineStr">
+      <c r="H8" s="27" t="inlineStr">
         <is>
           <t>UPGRADED from earlier 'too big': textile/PVA heritage = real PVA know-how; family-owned/agile. Best blend of PVA expertise + small-batch fit. (336) 885-5131.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Columbus Chemical (CCI)</t>
         </is>
       </c>
-      <c r="B9" s="31" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>Columbus, WI / Phoenix, AZ</t>
         </is>
       </c>
-      <c r="C9" s="31" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="D9" s="31" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>Yes — heating/cooling</t>
         </is>
       </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>20 L - 20,000 L (~5 gal floor)</t>
         </is>
       </c>
-      <c r="F9" s="31" t="inlineStr">
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>Excellent — lowest floor, widest range</t>
         </is>
       </c>
-      <c r="G9" s="34" t="inlineStr">
+      <c r="G9" s="38" t="inlineStr">
         <is>
           <t>STRONG</t>
         </is>
       </c>
-      <c r="H9" s="31" t="inlineStr">
+      <c r="H9" s="27" t="inlineStr">
         <is>
           <t>In-house lab, ISO 9001. Widest batch range = least shelf-life waste; can scale if demand grows.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>CORECHEM</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>Knoxville, TN</t>
         </is>
       </c>
-      <c r="C10" s="31" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="D10" s="31" t="inlineStr">
+      <c r="D10" s="27" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="E10" s="31" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>smallest tank ~250 gal (~4.5 drums)</t>
         </is>
       </c>
-      <c r="F10" s="31" t="inlineStr">
+      <c r="F10" s="27" t="inlineStr">
         <is>
           <t>CAUTION — 250-gal min may overshoot 18-day shelf life</t>
         </is>
       </c>
-      <c r="G10" s="35" t="inlineStr">
+      <c r="G10" s="39" t="inlineStr">
         <is>
           <t>CAUTION</t>
         </is>
       </c>
-      <c r="H10" s="31" t="inlineStr">
+      <c r="H10" s="27" t="inlineStr">
         <is>
           <t>Low-MOQ, start-up-friendly, family-owned. ASK about PARTIAL batches: a full 250-gal batch = ~4.5 drums but you can only use ~2 within 18 days.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>Northstar Chemical</t>
         </is>
       </c>
-      <c r="B11" s="31" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>Charlotte, NC</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>Backup</t>
         </is>
       </c>
-      <c r="D11" s="31" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>Confirm</t>
         </is>
       </c>
-      <c r="E11" s="31" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>unknown (small custom/toll)</t>
         </is>
       </c>
-      <c r="F11" s="31" t="inlineStr">
+      <c r="F11" s="27" t="inlineStr">
         <is>
           <t>Likely good — verify</t>
         </is>
       </c>
-      <c r="G11" s="33" t="inlineStr">
+      <c r="G11" s="37" t="inlineStr">
         <is>
           <t>LIKELY GOOD</t>
         </is>
       </c>
-      <c r="H11" s="31" t="inlineStr">
+      <c r="H11" s="27" t="inlineStr">
         <is>
           <t>Smaller dry-to-liquid custom/toll blender. (800) 570-0204.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>TECHNICAL ADVISOR — won't supply at this volume, but free expert call</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="inlineStr">
+      <c r="A13" s="27" t="inlineStr">
         <is>
           <t>Sekisui Specialty Chemicals</t>
         </is>
       </c>
-      <c r="B13" s="31" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>Calvert City, KY / Pasadena, TX</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>Advisor only</t>
         </is>
       </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr">
+      <c r="E13" s="27" t="inlineStr">
         <is>
           <t>n/a (producer, bulk only)</t>
         </is>
       </c>
-      <c r="F13" s="31" t="inlineStr">
+      <c r="F13" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G13" s="36" t="inlineStr">
+      <c r="G13" s="40" t="inlineStr">
         <is>
           <t>N/A — advisor</t>
         </is>
       </c>
-      <c r="H13" s="31" t="inlineStr">
+      <c r="H13" s="27" t="inlineStr">
         <is>
           <t>Largest US PVOH (Selvol) producer. Free Tech Services call on grade selection + cook procedure. +1 855 436 8683.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="36" t="inlineStr">
         <is>
           <t>DROPPED — too large / MOQ mismatch for ~1 drum/wk</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="inlineStr">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>Goulston Technologies</t>
         </is>
       </c>
-      <c r="B15" s="31" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>Monroe, NC</t>
         </is>
       </c>
-      <c r="C15" s="31" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D15" s="31" t="inlineStr">
+      <c r="D15" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="31" t="inlineStr">
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>large</t>
         </is>
       </c>
-      <c r="F15" s="31" t="inlineStr">
+      <c r="F15" s="27" t="inlineStr">
         <is>
           <t>Too big</t>
         </is>
       </c>
-      <c r="G15" s="37" t="inlineStr">
+      <c r="G15" s="41" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H15" s="31" t="inlineStr">
+      <c r="H15" s="27" t="inlineStr">
         <is>
           <t>Large textile chemical maker. 704-289-6464.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>3V Sigma USA</t>
         </is>
       </c>
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Georgetown, SC</t>
         </is>
       </c>
-      <c r="C16" s="31" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D16" s="31" t="inlineStr">
+      <c r="D16" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="31" t="inlineStr">
+      <c r="E16" s="27" t="inlineStr">
         <is>
           <t>large</t>
         </is>
       </c>
-      <c r="F16" s="31" t="inlineStr">
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>Too big</t>
         </is>
       </c>
-      <c r="G16" s="37" t="inlineStr">
+      <c r="G16" s="41" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H16" s="31" t="inlineStr">
+      <c r="H16" s="27" t="inlineStr">
         <is>
           <t>Large specialty chemical producer.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>Royal Chemical</t>
         </is>
       </c>
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>Twinsburg, OH (+5 sites)</t>
         </is>
       </c>
-      <c r="C17" s="31" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D17" s="31" t="inlineStr">
+      <c r="D17" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="31" t="inlineStr">
+      <c r="E17" s="27" t="inlineStr">
         <is>
           <t>220-gal liquid MOQ (~4 drums)</t>
         </is>
       </c>
-      <c r="F17" s="31" t="inlineStr">
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>MOQ overshoots shelf life</t>
         </is>
       </c>
-      <c r="G17" s="37" t="inlineStr">
+      <c r="G17" s="41" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H17" s="31" t="inlineStr">
+      <c r="H17" s="27" t="inlineStr">
         <is>
           <t>220-gal min = ~4 drums = ~4 wks supply &gt; 18-day shelf life.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="31" t="inlineStr">
+      <c r="A18" s="27" t="inlineStr">
         <is>
           <t>Columbia Chemical</t>
         </is>
       </c>
-      <c r="B18" s="31" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>Brunswick, OH</t>
         </is>
       </c>
-      <c r="C18" s="31" t="inlineStr">
+      <c r="C18" s="27" t="inlineStr">
         <is>
           <t>Dropped</t>
         </is>
       </c>
-      <c r="D18" s="31" t="inlineStr">
+      <c r="D18" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E18" s="31" t="inlineStr">
+      <c r="E18" s="27" t="inlineStr">
         <is>
           <t>large</t>
         </is>
       </c>
-      <c r="F18" s="31" t="inlineStr">
+      <c r="F18" s="27" t="inlineStr">
         <is>
           <t>Too big / mismatch</t>
         </is>
       </c>
-      <c r="G18" s="37" t="inlineStr">
+      <c r="G18" s="41" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H18" s="31" t="inlineStr"/>
+      <c r="H18" s="27" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="36" t="inlineStr">
         <is>
           <t>ELIMINATED — failed the 90-95 C cook</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>ArroChem</t>
         </is>
       </c>
-      <c r="B20" s="31" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>Mt. Holly, NC</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>ELIMINATED</t>
         </is>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>85 C ceiling — FAILS</t>
         </is>
       </c>
-      <c r="E20" s="31" t="inlineStr">
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>55 gal (would have fit)</t>
         </is>
       </c>
-      <c r="F20" s="31" t="inlineStr">
+      <c r="F20" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G20" s="37" t="inlineStr">
+      <c r="G20" s="41" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H20" s="31" t="inlineStr">
+      <c r="H20" s="27" t="inlineStr">
         <is>
           <t>Volume fit was perfect (55-gal floor) but can't reach the 90-95 C cook.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="A21" s="27" t="inlineStr">
         <is>
           <t>ILC Dover</t>
         </is>
       </c>
-      <c r="B21" s="31" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>Frederica, DE</t>
         </is>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>ELIMINATED</t>
         </is>
       </c>
-      <c r="D21" s="31" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>Can't reach 95 C</t>
         </is>
       </c>
-      <c r="E21" s="31" t="inlineStr">
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>n/a (equipment firm)</t>
         </is>
       </c>
-      <c r="F21" s="31" t="inlineStr">
+      <c r="F21" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G21" s="37" t="inlineStr">
+      <c r="G21" s="41" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H21" s="31" t="inlineStr">
+      <c r="H21" s="27" t="inlineStr">
         <is>
           <t>Wrong category (Ingersoll Rand containment/equipment) + heating fail. Close out.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="32" t="inlineStr">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>RAW RESIN PATH — reference only (supply Selvol resin, not the liquid blend)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t>Brenntag</t>
         </is>
       </c>
-      <c r="B23" s="31" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>US-wide</t>
         </is>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="D23" s="31" t="inlineStr">
+      <c r="D23" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E23" s="31" t="inlineStr">
+      <c r="E23" s="27" t="inlineStr">
         <is>
           <t>single drums (core)</t>
         </is>
       </c>
-      <c r="F23" s="31" t="inlineStr">
+      <c r="F23" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G23" s="36" t="inlineStr">
+      <c r="G23" s="40" t="inlineStr">
         <is>
           <t>N/A — distributor</t>
         </is>
       </c>
-      <c r="H23" s="31" t="inlineStr">
+      <c r="H23" s="27" t="inlineStr">
         <is>
           <t>Already lists Sekisui Selvol → easiest source of genuine resin in drums if a blender needs it supplied.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="31" t="inlineStr">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>Tilley / Palmer Holland</t>
         </is>
       </c>
-      <c r="B24" s="31" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>Baltimore, MD / Westlake, OH</t>
         </is>
       </c>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="D24" s="31" t="inlineStr">
+      <c r="D24" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="E24" s="31" t="inlineStr">
+      <c r="E24" s="27" t="inlineStr">
         <is>
           <t>drums</t>
         </is>
       </c>
-      <c r="F24" s="31" t="inlineStr">
+      <c r="F24" s="27" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="G24" s="36" t="inlineStr">
+      <c r="G24" s="40" t="inlineStr">
         <is>
           <t>N/A — distributor</t>
         </is>
       </c>
-      <c r="H24" s="31" t="inlineStr">
+      <c r="H24" s="27" t="inlineStr">
         <is>
           <t>Relationship-sized distributors; confirm they carry a PVA brand. Use only if sourcing raw resin.</t>
         </is>
@@ -2799,7 +3334,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2835,13 +3370,13 @@
           <t>Supplier</t>
         </is>
       </c>
-      <c r="C4" s="38" t="inlineStr">
+      <c r="C4" s="42" t="inlineStr">
         <is>
           <t>CJB Applied Technologies (Valdosta, GA)</t>
         </is>
       </c>
-      <c r="D4" s="39" t="n"/>
-      <c r="E4" s="40" t="n"/>
+      <c r="D4" s="43" t="n"/>
+      <c r="E4" s="44" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="17" t="inlineStr">
@@ -2849,13 +3384,13 @@
           <t>Phone / contact</t>
         </is>
       </c>
-      <c r="C5" s="38" t="inlineStr">
+      <c r="C5" s="42" t="inlineStr">
         <is>
           <t>(229) 588-7200  /  ____</t>
         </is>
       </c>
-      <c r="D5" s="39" t="n"/>
-      <c r="E5" s="40" t="n"/>
+      <c r="D5" s="43" t="n"/>
+      <c r="E5" s="44" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="17" t="inlineStr">
@@ -2863,13 +3398,13 @@
           <t>Date of call</t>
         </is>
       </c>
-      <c r="C6" s="38" t="inlineStr">
+      <c r="C6" s="42" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="D6" s="39" t="n"/>
-      <c r="E6" s="40" t="n"/>
+      <c r="D6" s="43" t="n"/>
+      <c r="E6" s="44" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="17" t="inlineStr">
@@ -2877,13 +3412,13 @@
           <t>Interviewer</t>
         </is>
       </c>
-      <c r="C7" s="38" t="inlineStr">
+      <c r="C7" s="42" t="inlineStr">
         <is>
           <t>Oscar P</t>
         </is>
       </c>
-      <c r="D7" s="39" t="n"/>
-      <c r="E7" s="40" t="n"/>
+      <c r="D7" s="43" t="n"/>
+      <c r="E7" s="44" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
@@ -2896,238 +3431,238 @@
       <c r="E9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="41" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Field</t>
         </is>
       </c>
-      <c r="C10" s="41" t="inlineStr">
+      <c r="C10" s="29" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
-      <c r="D10" s="41" t="inlineStr">
+      <c r="D10" s="29" t="inlineStr">
         <is>
           <t>Maps to</t>
         </is>
       </c>
-      <c r="E10" s="40" t="n"/>
+      <c r="E10" s="44" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="31" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>Holds 90-95 C cook 30-45 min? (Y/N)</t>
         </is>
       </c>
-      <c r="C11" s="42" t="inlineStr">
+      <c r="C11" s="45" t="inlineStr">
         <is>
           <t>YES — holds 45 min to 1 hr</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="46" t="inlineStr">
         <is>
           <t>HARD GATE — CLEARED</t>
         </is>
       </c>
-      <c r="E11" s="40" t="n"/>
+      <c r="E11" s="44" t="n"/>
     </row>
     <row r="12">
-      <c r="B12" s="31" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>Dissolves super-hydrolyzed HMW PVA? (Y/N)</t>
         </is>
       </c>
-      <c r="C12" s="42" t="inlineStr">
+      <c r="C12" s="45" t="inlineStr">
         <is>
           <t>YES — has prior experience</t>
         </is>
       </c>
-      <c r="D12" s="43" t="inlineStr">
+      <c r="D12" s="46" t="inlineStr">
         <is>
           <t>HARD GATE — CLEARED</t>
         </is>
       </c>
-      <c r="E12" s="40" t="n"/>
+      <c r="E12" s="44" t="n"/>
     </row>
     <row r="13">
-      <c r="B13" s="31" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>Min batch size (gal)</t>
         </is>
       </c>
-      <c r="C13" s="42" t="inlineStr">
+      <c r="C13" s="45" t="inlineStr">
         <is>
           <t>40 gal min</t>
         </is>
       </c>
-      <c r="D13" s="43" t="inlineStr">
+      <c r="D13" s="46" t="inlineStr">
         <is>
           <t>Inputs!MinBatch + shelf-life fit</t>
         </is>
       </c>
-      <c r="E13" s="40" t="n"/>
+      <c r="E13" s="44" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="31" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Will do partial / short batches? (Y/N)</t>
         </is>
       </c>
-      <c r="C14" s="42" t="inlineStr">
+      <c r="C14" s="45" t="inlineStr">
         <is>
           <t>YES — down to 40 gal; can lab-batch</t>
         </is>
       </c>
-      <c r="D14" s="43" t="inlineStr">
+      <c r="D14" s="46" t="inlineStr">
         <is>
           <t>18-day shelf-life fit</t>
         </is>
       </c>
-      <c r="E14" s="40" t="n"/>
+      <c r="E14" s="44" t="n"/>
     </row>
     <row r="15">
-      <c r="B15" s="31" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>MOQ per order (drums)</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C15" s="45" t="inlineStr">
         <is>
           <t>100 gal (~2 drums); will do 55 gal (1 drum)</t>
         </is>
       </c>
-      <c r="D15" s="43" t="inlineStr">
+      <c r="D15" s="46" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E15" s="40" t="n"/>
+      <c r="E15" s="44" t="n"/>
     </row>
     <row r="16">
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>Price/drum — Option A, base ($)</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C16" s="45" t="inlineStr">
         <is>
           <t>NOT yet quoted (pending NDA + spec)</t>
         </is>
       </c>
-      <c r="D16" s="43" t="inlineStr">
+      <c r="D16" s="46" t="inlineStr">
         <is>
           <t>Price Sensitivity input</t>
         </is>
       </c>
-      <c r="E16" s="40" t="n"/>
+      <c r="E16" s="44" t="n"/>
     </row>
     <row r="17">
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>Price/drum — Option B, compounded ($)</t>
         </is>
       </c>
-      <c r="C17" s="42" t="inlineStr">
+      <c r="C17" s="45" t="inlineStr">
         <is>
           <t>NOT yet quoted</t>
         </is>
       </c>
-      <c r="D17" s="43" t="inlineStr">
+      <c r="D17" s="46" t="inlineStr">
         <is>
           <t>Price Sensitivity input</t>
         </is>
       </c>
-      <c r="E17" s="40" t="n"/>
+      <c r="E17" s="44" t="n"/>
     </row>
     <row r="18">
-      <c r="B18" s="31" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>Lead time PO-&gt;delivery (days)</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C18" s="45" t="inlineStr">
         <is>
           <t>3-4 days, or overnight</t>
         </is>
       </c>
-      <c r="D18" s="43" t="inlineStr">
+      <c r="D18" s="46" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E18" s="40" t="n"/>
+      <c r="E18" s="44" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="31" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>Qualification sample qty &amp; cost</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="45" t="inlineStr">
         <is>
           <t>(not stated on call)</t>
         </is>
       </c>
-      <c r="D19" s="43" t="inlineStr">
+      <c r="D19" s="46" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E19" s="40" t="n"/>
+      <c r="E19" s="44" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="31" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>ISO 9001 / 13485? (which)</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C20" s="45" t="inlineStr">
         <is>
           <t>We don't require it</t>
         </is>
       </c>
-      <c r="D20" s="43" t="inlineStr">
+      <c r="D20" s="46" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E20" s="40" t="n"/>
+      <c r="E20" s="44" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="31" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>Prior PVA / HMW polymer experience? (Y/N)</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C21" s="45" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D21" s="43" t="inlineStr">
+      <c r="D21" s="46" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E21" s="40" t="n"/>
+      <c r="E21" s="44" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="31" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>NDA status</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C22" s="45" t="inlineStr">
         <is>
           <t>Needed on process before full spec shared</t>
         </is>
       </c>
-      <c r="D22" s="43" t="inlineStr">
+      <c r="D22" s="46" t="inlineStr">
         <is>
           <t>Roster</t>
         </is>
       </c>
-      <c r="E22" s="40" t="n"/>
+      <c r="E22" s="44" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="3" t="inlineStr">
@@ -3140,492 +3675,492 @@
       <c r="E24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="41" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B25" s="41" t="inlineStr">
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C25" s="41" t="inlineStr">
+      <c r="C25" s="29" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
-      <c r="D25" s="41" t="inlineStr">
+      <c r="D25" s="29" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
       </c>
-      <c r="E25" s="40" t="n"/>
+      <c r="E25" s="44" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="44" t="n"/>
+      <c r="A26" s="47" t="n"/>
       <c r="B26" s="4" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="45" t="n">
+      <c r="A27" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="31" t="inlineStr">
+      <c r="B27" s="27" t="inlineStr">
         <is>
           <t>Can you heat a FULL batch to 90-95 C (194-203 F) and HOLD 30-45 min under steady agitation? Our cook requires it.</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C27" s="45" t="inlineStr">
         <is>
           <t>Yes — holds 45 min to 1 hr</t>
         </is>
       </c>
-      <c r="D27" s="46" t="inlineStr">
+      <c r="D27" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E27" s="40" t="n"/>
+      <c r="E27" s="44" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="45" t="n">
+      <c r="A28" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="B28" s="31" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>Jacketed, temperature-controlled tank; 316L stainless contact surfaces?</t>
         </is>
       </c>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="C28" s="45" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D28" s="46" t="inlineStr">
+      <c r="D28" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E28" s="40" t="n"/>
+      <c r="E28" s="44" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="45" t="n">
+      <c r="A29" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="B29" s="31" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>Variable-speed agitation able to dissolve high-MW super-hydrolyzed PVA with NO fisheyes / gels?</t>
         </is>
       </c>
-      <c r="C29" s="42" t="inlineStr">
+      <c r="C29" s="45" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D29" s="46" t="inlineStr">
+      <c r="D29" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E29" s="40" t="n"/>
+      <c r="E29" s="44" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="45" t="n">
+      <c r="A30" s="48" t="n">
         <v>4</v>
       </c>
-      <c r="B30" s="31" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>Cooling capability to bring batch to &lt;=40 C?</t>
         </is>
       </c>
-      <c r="C30" s="42" t="inlineStr">
+      <c r="C30" s="45" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D30" s="46" t="inlineStr">
+      <c r="D30" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E30" s="40" t="n"/>
+      <c r="E30" s="44" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="45" t="n">
+      <c r="A31" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="B31" s="31" t="inlineStr">
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>Have you dissolved PVA or similar high-MW water-soluble polymers before? Examples?</t>
         </is>
       </c>
-      <c r="C31" s="42" t="inlineStr">
+      <c r="C31" s="45" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="D31" s="46" t="inlineStr">
+      <c r="D31" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E31" s="40" t="n"/>
+      <c r="E31" s="44" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="44" t="n"/>
+      <c r="A32" s="47" t="n"/>
       <c r="B32" s="4" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="45" t="n">
+      <c r="A33" s="48" t="n">
         <v>6</v>
       </c>
-      <c r="B33" s="31" t="inlineStr">
+      <c r="B33" s="27" t="inlineStr">
         <is>
           <t>Smallest batch you'll run? Will you do PARTIAL / short batches (~1-2 drums = 55-110 gal)?</t>
         </is>
       </c>
-      <c r="C33" s="42" t="inlineStr">
+      <c r="C33" s="45" t="inlineStr">
         <is>
           <t>40 gallons minimum</t>
         </is>
       </c>
-      <c r="D33" s="46" t="inlineStr">
+      <c r="D33" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E33" s="40" t="n"/>
+      <c r="E33" s="44" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="45" t="n">
+      <c r="A34" s="48" t="n">
         <v>7</v>
       </c>
-      <c r="B34" s="31" t="inlineStr">
+      <c r="B34" s="27" t="inlineStr">
         <is>
           <t>MOQ per order and standard batch size?</t>
         </is>
       </c>
-      <c r="C34" s="42" t="inlineStr">
+      <c r="C34" s="45" t="inlineStr">
         <is>
           <t>100 gal; could do 55 gal</t>
         </is>
       </c>
-      <c r="D34" s="46" t="inlineStr">
+      <c r="D34" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E34" s="40" t="n"/>
+      <c r="E34" s="44" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="45" t="n">
+      <c r="A35" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="B35" s="31" t="inlineStr">
+      <c r="B35" s="27" t="inlineStr">
         <is>
           <t>Can you make-to-order on a ~weekly cadence? (18-day shelf life — we cannot stockpile.)</t>
         </is>
       </c>
-      <c r="C35" s="42" t="inlineStr">
+      <c r="C35" s="45" t="inlineStr">
         <is>
           <t>Yes — able to lab batch</t>
         </is>
       </c>
-      <c r="D35" s="46" t="inlineStr">
+      <c r="D35" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E35" s="40" t="n"/>
+      <c r="E35" s="44" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="44" t="n"/>
+      <c r="A36" s="47" t="n"/>
       <c r="B36" s="4" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="45" t="n">
+      <c r="A37" s="48" t="n">
         <v>9</v>
       </c>
-      <c r="B37" s="31" t="inlineStr">
+      <c r="B37" s="27" t="inlineStr">
         <is>
           <t>Comfortable running OUR supplied process: charge water -&gt; add resin + NaCl + pigments -&gt; heat/hold 90-95 C -&gt; add Proxel BD20 hot in final 10 min -&gt; filter 200 micron -&gt; drum?</t>
         </is>
       </c>
-      <c r="C37" s="42" t="inlineStr">
+      <c r="C37" s="45" t="inlineStr">
         <is>
           <t>(not covered — confirm w/ full spec)</t>
         </is>
       </c>
-      <c r="D37" s="46" t="inlineStr">
+      <c r="D37" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E37" s="40" t="n"/>
+      <c r="E37" s="44" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="45" t="n">
+      <c r="A38" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="B38" s="31" t="inlineStr">
+      <c r="B38" s="27" t="inlineStr">
         <is>
           <t>Filtration to 200 micron (100 mesh or finer)?</t>
         </is>
       </c>
-      <c r="C38" s="42" t="inlineStr">
+      <c r="C38" s="45" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D38" s="46" t="inlineStr">
+      <c r="D38" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E38" s="40" t="n"/>
+      <c r="E38" s="44" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="45" t="n">
+      <c r="A39" s="48" t="n">
         <v>11</v>
       </c>
-      <c r="B39" s="31" t="inlineStr">
+      <c r="B39" s="27" t="inlineStr">
         <is>
           <t>Your ex-Lonza formulator — any input on Proxel BD20 addition point / order / dosing?</t>
         </is>
       </c>
-      <c r="C39" s="42" t="inlineStr">
+      <c r="C39" s="45" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D39" s="46" t="inlineStr">
+      <c r="D39" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E39" s="40" t="n"/>
+      <c r="E39" s="44" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="45" t="n">
+      <c r="A40" s="48" t="n">
         <v>12</v>
       </c>
-      <c r="B40" s="31" t="inlineStr">
+      <c r="B40" s="27" t="inlineStr">
         <is>
           <t>Will you source raw materials to spec (Selvol S-1551F-D or equivalent) or do we supply the resin?</t>
         </is>
       </c>
-      <c r="C40" s="42" t="inlineStr">
+      <c r="C40" s="45" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D40" s="46" t="inlineStr">
+      <c r="D40" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E40" s="40" t="n"/>
+      <c r="E40" s="44" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="44" t="n"/>
+      <c r="A41" s="47" t="n"/>
       <c r="B41" s="4" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="45" t="n">
+      <c r="A42" s="48" t="n">
         <v>13</v>
       </c>
-      <c r="B42" s="31" t="inlineStr">
+      <c r="B42" s="27" t="inlineStr">
         <is>
           <t>55-gallon drum fill? 275-gal IBC totes optional?</t>
         </is>
       </c>
-      <c r="C42" s="42" t="inlineStr">
+      <c r="C42" s="45" t="inlineStr">
         <is>
           <t>Packaging is flexible</t>
         </is>
       </c>
-      <c r="D42" s="46" t="inlineStr">
+      <c r="D42" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E42" s="40" t="n"/>
+      <c r="E42" s="44" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="45" t="n">
+      <c r="A43" s="48" t="n">
         <v>14</v>
       </c>
-      <c r="B43" s="31" t="inlineStr">
+      <c r="B43" s="27" t="inlineStr">
         <is>
           <t>Protect-from-freezing handling in shipping/storage?</t>
         </is>
       </c>
-      <c r="C43" s="42" t="inlineStr">
+      <c r="C43" s="45" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D43" s="46" t="inlineStr">
+      <c r="D43" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E43" s="40" t="n"/>
+      <c r="E43" s="44" t="n"/>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="45" t="n">
+      <c r="A44" s="48" t="n">
         <v>15</v>
       </c>
-      <c r="B44" s="31" t="inlineStr">
+      <c r="B44" s="27" t="inlineStr">
         <is>
           <t>Shipping from GA to us — lead time &amp; freight cost?</t>
         </is>
       </c>
-      <c r="C44" s="42" t="inlineStr">
+      <c r="C44" s="45" t="inlineStr">
         <is>
           <t>Lead time ~3-4 days, or overnight</t>
         </is>
       </c>
-      <c r="D44" s="46" t="inlineStr">
+      <c r="D44" s="49" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="E44" s="40" t="n"/>
+      <c r="E44" s="44" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="44" t="n"/>
+      <c r="A45" s="47" t="n"/>
       <c r="B45" s="4" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="45" t="n">
+      <c r="A46" s="48" t="n">
         <v>16</v>
       </c>
-      <c r="B46" s="31" t="inlineStr">
+      <c r="B46" s="27" t="inlineStr">
         <is>
           <t>CoC every shipment with lot#, production date, %TS, final pH, Brookfield viscosity (spindle #3, 10 RPM, 25 C)?</t>
         </is>
       </c>
-      <c r="C46" s="42" t="inlineStr">
+      <c r="C46" s="45" t="inlineStr">
         <is>
           <t>(not covered — confirm)</t>
         </is>
       </c>
-      <c r="D46" s="46" t="inlineStr">
+      <c r="D46" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E46" s="40" t="n"/>
+      <c r="E46" s="44" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="45" t="n">
+      <c r="A47" s="48" t="n">
         <v>17</v>
       </c>
-      <c r="B47" s="31" t="inlineStr">
+      <c r="B47" s="27" t="inlineStr">
         <is>
           <t>Typical batch-to-batch variability on viscosity &amp; pH for similar solutions?</t>
         </is>
       </c>
-      <c r="C47" s="42" t="inlineStr">
+      <c r="C47" s="45" t="inlineStr">
         <is>
           <t>(not covered)</t>
         </is>
       </c>
-      <c r="D47" s="46" t="inlineStr">
+      <c r="D47" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E47" s="40" t="n"/>
+      <c r="E47" s="44" t="n"/>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="45" t="n">
+      <c r="A48" s="48" t="n">
         <v>18</v>
       </c>
-      <c r="B48" s="31" t="inlineStr">
+      <c r="B48" s="27" t="inlineStr">
         <is>
           <t>Certifications — ISO 9001 minimum; ISO 13485 if available?</t>
         </is>
       </c>
-      <c r="C48" s="42" t="inlineStr">
+      <c r="C48" s="45" t="inlineStr">
         <is>
           <t>We don't require ISO certs</t>
         </is>
       </c>
-      <c r="D48" s="46" t="inlineStr">
+      <c r="D48" s="49" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="E48" s="40" t="n"/>
+      <c r="E48" s="44" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="44" t="n"/>
+      <c r="A49" s="47" t="n"/>
       <c r="B49" s="4" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="45" t="n">
+      <c r="A50" s="48" t="n">
         <v>19</v>
       </c>
-      <c r="B50" s="31" t="inlineStr">
+      <c r="B50" s="27" t="inlineStr">
         <is>
           <t>Quote BOTH Option A (base PVA solution) and Option B (full compounded w/ NaCl + pigments)?</t>
         </is>
       </c>
-      <c r="C50" s="42" t="inlineStr">
+      <c r="C50" s="45" t="inlineStr">
         <is>
           <t>(not yet — needs spec/NDA)</t>
         </is>
       </c>
-      <c r="D50" s="46" t="inlineStr">
+      <c r="D50" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E50" s="40" t="n"/>
+      <c r="E50" s="44" t="n"/>
     </row>
     <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="45" t="n">
+      <c r="A51" s="48" t="n">
         <v>20</v>
       </c>
-      <c r="B51" s="31" t="inlineStr">
+      <c r="B51" s="27" t="inlineStr">
         <is>
           <t>Per-drum pricing — we'll run this as a recurring rotation, ~1 drum/wk slice, ~30-38 drums/yr. Volume-agnostic per-drum quote?</t>
         </is>
       </c>
-      <c r="C51" s="42" t="inlineStr">
+      <c r="C51" s="45" t="inlineStr">
         <is>
           <t>(not yet quoted)</t>
         </is>
       </c>
-      <c r="D51" s="46" t="inlineStr">
+      <c r="D51" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E51" s="40" t="n"/>
+      <c r="E51" s="44" t="n"/>
     </row>
     <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="45" t="n">
+      <c r="A52" s="48" t="n">
         <v>21</v>
       </c>
-      <c r="B52" s="31" t="inlineStr">
+      <c r="B52" s="27" t="inlineStr">
         <is>
           <t>Lead time, qualification sample cost, and NDA needed before we share the full spec?</t>
         </is>
       </c>
-      <c r="C52" s="42" t="inlineStr">
+      <c r="C52" s="45" t="inlineStr">
         <is>
           <t>NDA needed on process</t>
         </is>
       </c>
-      <c r="D52" s="46" t="inlineStr">
+      <c r="D52" s="49" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="E52" s="40" t="n"/>
+      <c r="E52" s="44" t="n"/>
     </row>
     <row r="54">
       <c r="B54" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Apply hard cap: 2nd source gets no more than 1 drum/week
- Model: allocation labeled HARD CAP=1; cost matrix + split notes flag
  35% (~1 drum/wk) as the cap and 50% as reference-only
- Slides: cost table drops over-cap row; pricing slide swaps the 2-drum
  batch lever for steady-weekly-PO (capped at 1/wk); cadence slide
  reframed to weekly single-drum as recommended; summary range -> ~$0-24k
- Report: cost table + ranges updated for the cap

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LkE2ZRYs3PLyj8XHTsU3i4
</commit_message>
<xml_diff>
--- a/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
+++ b/PVA second supplier initiative/PVA_Second_Source_Pricing_Model.xlsx
@@ -911,7 +911,7 @@
     <row r="18">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>2nd-source allocation (drums / week)  &lt;-- SCENARIO LEVER</t>
+          <t>2nd-source allocation (drums / week)  &lt;-- HARD CAP = 1</t>
         </is>
       </c>
       <c r="C18" s="13" t="n">
@@ -919,7 +919,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Scenario lever, NOT a decision. Change to explore. 1 drum/wk shown only as an example = ~35% of volume.</t>
+          <t>HARD CAP: no more than 1 drum/week to this supplier (~35% of volume, ~52 drums/yr). Do not exceed 1.</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Each row is a SCENARIO (nothing decided). 'Δ vs all-SNP' = the annual cost of keeping a second source at that split, assuming SNP HOLDS its price. For SNP-raises-price cases see the 'SNP Re-pricing Risk' and 'Cost of 2nd Source' tabs.</t>
+          <t>Each row is a SCENARIO. 'Δ vs all-SNP' = annual cost of a second source at that split (SNP price held). CAP: this supplier gets no more than 1 drum/wk (~35%); the 50% row is reference only. SNP-raises-price cases: see 'SNP Re-pricing Risk' and 'Cost of 2nd Source' tabs.</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Premium = baseline x [ allocation x (2nd-source price premium) + retained x (SNP surcharge) ].   Note: 1 drum/wk ~= 35% of volume.</t>
+          <t>Premium = baseline x [ allocation x (2nd-source price premium) + retained x (SNP surcharge) ].   HARD CAP: 1 drum/wk (~35%) is the most this supplier gets; the 50% row is reference only.</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2203,7 @@
     <row r="10">
       <c r="A10" s="30" t="inlineStr">
         <is>
-          <t>35% (~1 drum/wk)</t>
+          <t>35% (~1 drum/wk — CAP)</t>
         </is>
       </c>
       <c r="B10" s="31">
@@ -2226,7 +2226,7 @@
     <row r="11">
       <c r="A11" s="30" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>50% (&gt; cap, ref)</t>
         </is>
       </c>
       <c r="B11" s="31">
@@ -2352,7 +2352,7 @@
     <row r="18">
       <c r="A18" s="30" t="inlineStr">
         <is>
-          <t>35% (~1 drum/wk)</t>
+          <t>35% (~1 drum/wk — CAP)</t>
         </is>
       </c>
       <c r="B18" s="31">
@@ -2375,7 +2375,7 @@
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>50% (&gt; cap, ref)</t>
         </is>
       </c>
       <c r="B19" s="31">
@@ -2501,7 +2501,7 @@
     <row r="26">
       <c r="A26" s="30" t="inlineStr">
         <is>
-          <t>35% (~1 drum/wk)</t>
+          <t>35% (~1 drum/wk — CAP)</t>
         </is>
       </c>
       <c r="B26" s="31">
@@ -2524,7 +2524,7 @@
     <row r="27">
       <c r="A27" s="30" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>50% (&gt; cap, ref)</t>
         </is>
       </c>
       <c r="B27" s="31">

</xml_diff>